<commit_message>
Spreadsheet updates 9.15.2026 for November26 PPP
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E04CC331-D618-4E14-937C-E986254297CF}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{984C8042-7220-4C79-8C52-332B358F0FE4}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPP Projects" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="261">
   <si>
     <t>1st Review</t>
   </si>
@@ -795,7 +795,29 @@
     <t>Sent for Final Signature to District</t>
   </si>
   <si>
-    <t>Plans Signed</t>
+    <t>9/112026</t>
+  </si>
+  <si>
+    <t>Send to District for the Sign</t>
+  </si>
+  <si>
+    <t>Emailed district to add SP and sign the plan 9.11.26</t>
+  </si>
+  <si>
+    <t>Emailed district to add two SPs and minor correction  9.11.26</t>
+  </si>
+  <si>
+    <t>Emailed to District for 3rd Revie on 9.1..2026</t>
+  </si>
+  <si>
+    <t>Emailed district to add SP&amp; minor c for 3rd Review on 9.11.26
+Emailed Sharon with the submission for her 4th Review 9.14.2026</t>
+  </si>
+  <si>
+    <t>Emailed sharon for final review on 9.14.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emailed sent to SB </t>
   </si>
 </sst>
 </file>
@@ -1094,6 +1116,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PPPProjectsTable" displayName="PPPProjectsTable" ref="A1:AK52" totalsRowShown="0">
   <autoFilter ref="A1:AK52" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -1546,12 +1572,26 @@
       <c r="V2" s="20">
         <v>46273</v>
       </c>
-      <c r="W2" s="20"/>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
-      <c r="AA2" s="24"/>
+      <c r="W2" s="20">
+        <v>46274</v>
+      </c>
+      <c r="X2" s="20">
+        <v>46276</v>
+      </c>
+      <c r="Y2" s="20">
+        <v>46276</v>
+      </c>
+      <c r="Z2" s="20">
+        <v>46276</v>
+      </c>
+      <c r="AA2" s="24" t="s">
+        <v>253</v>
+      </c>
       <c r="AB2" s="24"/>
-      <c r="AK2" s="20"/>
+      <c r="AC2" s="20"/>
+      <c r="AK2" s="20" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="3" spans="1:37">
       <c r="A3" s="11" t="s">
@@ -1629,10 +1669,16 @@
       <c r="Y3" s="20">
         <v>46268</v>
       </c>
-      <c r="AA3" s="24"/>
+      <c r="Z3" s="20">
+        <v>46276</v>
+      </c>
+      <c r="AA3" s="24">
+        <v>46276</v>
+      </c>
       <c r="AB3" s="24"/>
+      <c r="AC3" s="20"/>
       <c r="AK3" s="20" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:37">
@@ -1711,14 +1757,17 @@
       <c r="Y4" s="20">
         <v>46268</v>
       </c>
+      <c r="Z4" s="20">
+        <v>46273</v>
+      </c>
       <c r="AA4" s="24">
         <v>46273</v>
       </c>
       <c r="AB4" s="24">
         <v>46274</v>
       </c>
-      <c r="AK4" s="20" t="s">
-        <v>252</v>
+      <c r="AC4" s="20">
+        <v>46275</v>
       </c>
     </row>
     <row r="5" spans="1:37">
@@ -1770,10 +1819,18 @@
       <c r="P5" s="20">
         <v>46269</v>
       </c>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20"/>
-      <c r="T5" s="20"/>
+      <c r="Q5" s="20">
+        <v>46275</v>
+      </c>
+      <c r="R5" s="20">
+        <v>46275</v>
+      </c>
+      <c r="S5" s="20">
+        <v>46275</v>
+      </c>
+      <c r="T5" s="20">
+        <v>46276</v>
+      </c>
       <c r="U5" s="20"/>
       <c r="V5" s="20"/>
       <c r="W5" s="20"/>
@@ -1781,7 +1838,10 @@
       <c r="Y5" s="20"/>
       <c r="AA5" s="24"/>
       <c r="AB5" s="24"/>
-      <c r="AK5" s="26"/>
+      <c r="AC5" s="20"/>
+      <c r="AK5" s="26" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="6" spans="1:37">
       <c r="A6" s="11" t="s">
@@ -1851,7 +1911,10 @@
       <c r="Y6" s="20"/>
       <c r="AA6" s="24"/>
       <c r="AB6" s="24"/>
-      <c r="AK6" s="20"/>
+      <c r="AC6" s="20"/>
+      <c r="AK6" s="20" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="7" spans="1:37">
       <c r="A7" s="11" t="s">
@@ -1914,15 +1977,18 @@
       <c r="T7" s="20">
         <v>46274</v>
       </c>
-      <c r="U7" s="20"/>
+      <c r="U7" s="20">
+        <v>46276</v>
+      </c>
       <c r="V7" s="20"/>
       <c r="W7" s="20"/>
       <c r="X7" s="20"/>
       <c r="Y7" s="20"/>
       <c r="AA7" s="24"/>
       <c r="AB7" s="24"/>
+      <c r="AC7" s="20"/>
       <c r="AK7" s="20" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" spans="1:37">
@@ -1986,14 +2052,21 @@
       <c r="T8" s="20">
         <v>46269</v>
       </c>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
+      <c r="U8" s="20">
+        <v>46273</v>
+      </c>
+      <c r="V8" s="20">
+        <v>46279</v>
+      </c>
       <c r="W8" s="20"/>
       <c r="X8" s="20"/>
       <c r="Y8" s="20"/>
       <c r="AA8" s="24"/>
       <c r="AB8" s="24"/>
-      <c r="AK8" s="26"/>
+      <c r="AC8" s="20"/>
+      <c r="AK8" s="20" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="9" spans="1:37">
       <c r="A9" s="11" t="s">
@@ -2044,17 +2117,43 @@
       <c r="P9" s="20">
         <v>46268</v>
       </c>
-      <c r="Q9" s="20"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
-      <c r="T9" s="20"/>
-      <c r="U9" s="20"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="20"/>
-      <c r="Y9" s="20"/>
-      <c r="AA9" s="24"/>
+      <c r="Q9" s="20">
+        <v>46276</v>
+      </c>
+      <c r="R9" s="20">
+        <v>46276</v>
+      </c>
+      <c r="S9" s="20">
+        <v>46276</v>
+      </c>
+      <c r="T9" s="20">
+        <v>46276</v>
+      </c>
+      <c r="U9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="V9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="W9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="X9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="Y9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="Z9" s="20">
+        <v>46279</v>
+      </c>
+      <c r="AA9" s="24">
+        <v>46279</v>
+      </c>
       <c r="AB9" s="24"/>
+      <c r="AC9" s="20">
+        <v>46279</v>
+      </c>
       <c r="AK9" s="20"/>
     </row>
     <row r="10" spans="1:37">
@@ -2133,14 +2232,16 @@
       <c r="Y10" s="20">
         <v>46274</v>
       </c>
+      <c r="Z10" s="20">
+        <v>46276</v>
+      </c>
       <c r="AA10" s="24">
-        <v>46274</v>
-      </c>
-      <c r="AB10" s="24">
-        <v>46274</v>
-      </c>
+        <v>46279</v>
+      </c>
+      <c r="AB10" s="24"/>
+      <c r="AC10" s="20"/>
       <c r="AK10" s="20" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -2198,8 +2299,12 @@
       <c r="R11" s="20">
         <v>46273</v>
       </c>
-      <c r="S11" s="20"/>
-      <c r="T11" s="20"/>
+      <c r="S11" s="20">
+        <v>46274</v>
+      </c>
+      <c r="T11" s="20">
+        <v>46276</v>
+      </c>
       <c r="U11" s="20"/>
       <c r="V11" s="20"/>
       <c r="W11" s="20"/>
@@ -2207,7 +2312,10 @@
       <c r="Y11" s="20"/>
       <c r="AA11" s="24"/>
       <c r="AB11" s="24"/>
-      <c r="AK11" s="20"/>
+      <c r="AC11" s="20"/>
+      <c r="AK11" s="20" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="12" spans="1:37">
       <c r="A12" s="11" t="s">
@@ -2287,6 +2395,7 @@
       </c>
       <c r="AA12" s="24"/>
       <c r="AB12" s="24"/>
+      <c r="AC12" s="20"/>
       <c r="AK12" s="20" t="s">
         <v>252</v>
       </c>
@@ -2369,6 +2478,7 @@
       </c>
       <c r="AA13" s="24"/>
       <c r="AB13" s="25"/>
+      <c r="AC13" s="20"/>
       <c r="AK13" s="20" t="s">
         <v>251</v>
       </c>
@@ -2434,13 +2544,33 @@
       <c r="T14" s="20">
         <v>46274</v>
       </c>
-      <c r="U14" s="20"/>
-      <c r="V14" s="20"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="20"/>
-      <c r="Y14" s="20"/>
-      <c r="AA14" s="24"/>
-      <c r="AB14" s="24"/>
+      <c r="U14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="V14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="W14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="X14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="Y14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="Z14" s="20">
+        <v>46279</v>
+      </c>
+      <c r="AA14" s="24">
+        <v>46279</v>
+      </c>
+      <c r="AB14" s="24">
+        <v>46279</v>
+      </c>
+      <c r="AC14" s="20">
+        <v>46279</v>
+      </c>
       <c r="AK14" s="20"/>
     </row>
     <row r="15" spans="1:37">

</xml_diff>

<commit_message>
Spreadsheet updates 9.16.2026 for November26 PPP
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{984C8042-7220-4C79-8C52-332B358F0FE4}"/>
+  <xr:revisionPtr revIDLastSave="128" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E30F0BCE-EA77-4D0E-9C9D-69FBA6F1D9DE}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -807,17 +807,16 @@
     <t>Emailed district to add two SPs and minor correction  9.11.26</t>
   </si>
   <si>
-    <t>Emailed to District for 3rd Revie on 9.1..2026</t>
-  </si>
-  <si>
-    <t>Emailed district to add SP&amp; minor c for 3rd Review on 9.11.26
-Emailed Sharon with the submission for her 4th Review 9.14.2026</t>
-  </si>
-  <si>
     <t>Emailed sharon for final review on 9.14.26</t>
   </si>
   <si>
     <t xml:space="preserve">Emailed sent to SB </t>
+  </si>
+  <si>
+    <t>9/15/23026</t>
+  </si>
+  <si>
+    <t>Emailed to SB for 4th Review</t>
   </si>
 </sst>
 </file>
@@ -1831,8 +1830,12 @@
       <c r="T5" s="20">
         <v>46276</v>
       </c>
-      <c r="U5" s="20"/>
-      <c r="V5" s="20"/>
+      <c r="U5" s="20">
+        <v>46281</v>
+      </c>
+      <c r="V5" s="20">
+        <v>46281</v>
+      </c>
       <c r="W5" s="20"/>
       <c r="X5" s="20"/>
       <c r="Y5" s="20"/>
@@ -1904,8 +1907,12 @@
       <c r="T6" s="20">
         <v>46274</v>
       </c>
-      <c r="U6" s="20"/>
-      <c r="V6" s="20"/>
+      <c r="U6" s="20">
+        <v>46279</v>
+      </c>
+      <c r="V6" s="20">
+        <v>46279</v>
+      </c>
       <c r="W6" s="20"/>
       <c r="X6" s="20"/>
       <c r="Y6" s="20"/>
@@ -1913,7 +1920,7 @@
       <c r="AB6" s="24"/>
       <c r="AC6" s="20"/>
       <c r="AK6" s="20" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" spans="1:37">
@@ -1978,13 +1985,17 @@
         <v>46274</v>
       </c>
       <c r="U7" s="20">
-        <v>46276</v>
-      </c>
-      <c r="V7" s="20"/>
+        <v>46281</v>
+      </c>
+      <c r="V7" s="20">
+        <v>46281</v>
+      </c>
       <c r="W7" s="20"/>
       <c r="X7" s="20"/>
       <c r="Y7" s="20"/>
-      <c r="AA7" s="24"/>
+      <c r="AA7" s="24">
+        <v>9</v>
+      </c>
       <c r="AB7" s="24"/>
       <c r="AC7" s="20"/>
       <c r="AK7" s="20" t="s">
@@ -2058,15 +2069,26 @@
       <c r="V8" s="20">
         <v>46279</v>
       </c>
-      <c r="W8" s="20"/>
-      <c r="X8" s="20"/>
-      <c r="Y8" s="20"/>
-      <c r="AA8" s="24"/>
-      <c r="AB8" s="24"/>
+      <c r="W8" s="20">
+        <v>46280</v>
+      </c>
+      <c r="X8" s="20">
+        <v>46280</v>
+      </c>
+      <c r="Y8" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="Z8" s="20">
+        <v>46280</v>
+      </c>
+      <c r="AA8" s="24">
+        <v>46280</v>
+      </c>
+      <c r="AB8" s="24">
+        <v>46280</v>
+      </c>
       <c r="AC8" s="20"/>
-      <c r="AK8" s="20" t="s">
-        <v>258</v>
-      </c>
+      <c r="AK8" s="20"/>
     </row>
     <row r="9" spans="1:37">
       <c r="A9" s="11" t="s">
@@ -2241,7 +2263,7 @@
       <c r="AB10" s="24"/>
       <c r="AC10" s="20"/>
       <c r="AK10" s="20" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:37">
@@ -2314,7 +2336,7 @@
       <c r="AB11" s="24"/>
       <c r="AC11" s="20"/>
       <c r="AK11" s="20" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" spans="1:37">

</xml_diff>

<commit_message>
Update on PPP 2027 on 9.30.2026
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="144" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73EB935E-B469-482C-A8D5-4A10D5D99F6E}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED35B639-C39C-4866-90E0-42B1C21E1D9F}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PPP Projects" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="272">
   <si>
     <t>1st Review</t>
   </si>
@@ -618,9 +618,6 @@
     <t xml:space="preserve">2" Mill &amp; 2" Overlay </t>
   </si>
   <si>
-    <t>Level Up &amp; 2" Overlay w/ Patching; 2' Shoulders</t>
-  </si>
-  <si>
     <t xml:space="preserve">1.5" Overlay; 2' Shoulders </t>
   </si>
   <si>
@@ -789,31 +786,70 @@
     <t>090735</t>
   </si>
   <si>
-    <t>Email send to District for correction.</t>
-  </si>
-  <si>
-    <t>Sent for Final Signature to District</t>
-  </si>
-  <si>
     <t>9/112026</t>
   </si>
   <si>
-    <t>Send to District for the Sign</t>
-  </si>
-  <si>
-    <t>Emailed district to add SP and sign the plan 9.11.26</t>
-  </si>
-  <si>
-    <t>Emailed district to add two SPs and minor correction  9.11.26</t>
-  </si>
-  <si>
-    <t>Emailed sharon for final review on 9.14.26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emailed sent to SB </t>
-  </si>
-  <si>
-    <t>Emailed to SB for 4th Review</t>
+    <t>A20046</t>
+  </si>
+  <si>
+    <t>2” Overlay (Sec. 15 LM 0.00-1.796); FDR (Sec. 21 LM 1.796-2.253 &amp; Sec. 16 LM 0.00-9.650)</t>
+  </si>
+  <si>
+    <t>Dallas Co. Line - Hwy. 167 (S)</t>
+  </si>
+  <si>
+    <t>Level up &amp; UTBWC (Hwy. 167), UTBWC (Hwy. 167B)</t>
+  </si>
+  <si>
+    <t>10, 10B &amp;11B</t>
+  </si>
+  <si>
+    <t>A20045</t>
+  </si>
+  <si>
+    <t>A30053</t>
+  </si>
+  <si>
+    <t>A60069</t>
+  </si>
+  <si>
+    <t>A70051</t>
+  </si>
+  <si>
+    <t>A90036</t>
+  </si>
+  <si>
+    <t>Hwy. 133 – Hwy. 82 (S)</t>
+  </si>
+  <si>
+    <t>S. of Ogden - S. of Ashdown (S)</t>
+  </si>
+  <si>
+    <t>Shady Grove Rd. – Hwy. 270B</t>
+  </si>
+  <si>
+    <t>Gurdon - Nevada Co. Line (S)</t>
+  </si>
+  <si>
+    <t>N. of I-49 - Missouri State Line (Bella Vista) (S)</t>
+  </si>
+  <si>
+    <t>1" Level Up &amp; UTBWC</t>
+  </si>
+  <si>
+    <t>Ashley</t>
+  </si>
+  <si>
+    <t>Little River</t>
+  </si>
+  <si>
+    <t>Garland</t>
+  </si>
+  <si>
+    <t>9/258/2026</t>
+  </si>
+  <si>
+    <t>Waiting on correction from District</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1080,67 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2A31118A-900B-4722-A90B-8152F5F4035D}"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1114,19 +1210,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PPPProjectsTable" displayName="PPPProjectsTable" ref="A1:AK52" totalsRowShown="0">
-  <autoFilter ref="A1:AK52" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PPPProjectsTable" displayName="PPPProjectsTable" ref="A1:AK58" totalsRowShown="0">
+  <autoFilter ref="A1:AK58" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="37">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Job Number" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Job Number" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Project Description"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="District" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Route" dataDxfId="5"/>
-    <tableColumn id="36" xr3:uid="{B65E3A66-8F4F-4C7A-8EAC-7D6C80DA624C}" name="Section" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="County" dataDxfId="3"/>
-    <tableColumn id="37" xr3:uid="{91677106-A41F-4D5F-A2D6-7604E00D01E2}" name="Scope" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Letting Date" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="District" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Route" dataDxfId="11"/>
+    <tableColumn id="36" xr3:uid="{B65E3A66-8F4F-4C7A-8EAC-7D6C80DA624C}" name="Section" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="County" dataDxfId="9"/>
+    <tableColumn id="37" xr3:uid="{91677106-A41F-4D5F-A2D6-7604E00D01E2}" name="Scope" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Letting Date" dataDxfId="7"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Due to PM"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="1st Review Sent to SB" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="1st Review Sent to SB" dataDxfId="6"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="1st Review Returned from SB"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1st Review Sent to District"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="1st Review Returned from District"/>
@@ -1368,11 +1464,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AK52"/>
+  <dimension ref="A1:AK58"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="39.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.19921875" customWidth="1"/>
     <col min="3" max="3" width="10" style="11" customWidth="1"/>
     <col min="4" max="5" width="12" style="11" customWidth="1"/>
     <col min="6" max="6" width="19.8984375" style="11" bestFit="1" customWidth="1"/>
@@ -1578,7 +1674,7 @@
         <v>46276</v>
       </c>
       <c r="AA2" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="AB2" s="24">
         <v>46288</v>
@@ -1586,9 +1682,7 @@
       <c r="AC2" s="20">
         <v>46288</v>
       </c>
-      <c r="AK2" s="20" t="s">
-        <v>254</v>
-      </c>
+      <c r="AK2" s="20"/>
     </row>
     <row r="3" spans="1:37">
       <c r="A3" s="11" t="s">
@@ -1677,7 +1771,7 @@
       </c>
       <c r="AC3" s="20"/>
       <c r="AK3" s="20" t="s">
-        <v>255</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:37">
@@ -1857,9 +1951,7 @@
       <c r="AC5" s="20">
         <v>46282</v>
       </c>
-      <c r="AK5" s="25" t="s">
-        <v>256</v>
-      </c>
+      <c r="AK5" s="25"/>
     </row>
     <row r="6" spans="1:37">
       <c r="A6" s="11" t="s">
@@ -1949,9 +2041,7 @@
       <c r="AC6" s="20">
         <v>46287</v>
       </c>
-      <c r="AK6" s="20" t="s">
-        <v>259</v>
-      </c>
+      <c r="AK6" s="20"/>
     </row>
     <row r="7" spans="1:37">
       <c r="A7" s="11" t="s">
@@ -2041,9 +2131,7 @@
       <c r="AC7" s="20">
         <v>46287</v>
       </c>
-      <c r="AK7" s="20" t="s">
-        <v>255</v>
-      </c>
+      <c r="AK7" s="20"/>
     </row>
     <row r="8" spans="1:37">
       <c r="A8" s="11" t="s">
@@ -2313,9 +2401,7 @@
       <c r="AC10" s="20">
         <v>46288</v>
       </c>
-      <c r="AK10" s="20" t="s">
-        <v>257</v>
-      </c>
+      <c r="AK10" s="20"/>
     </row>
     <row r="11" spans="1:37">
       <c r="A11" s="11" t="s">
@@ -2390,15 +2476,22 @@
       <c r="X11" s="20">
         <v>46286</v>
       </c>
-      <c r="Y11" s="20"/>
+      <c r="Y11" s="20">
+        <v>46286</v>
+      </c>
+      <c r="Z11" s="20">
+        <v>46293</v>
+      </c>
       <c r="AA11" s="24">
         <v>46286</v>
       </c>
-      <c r="AB11" s="24"/>
-      <c r="AC11" s="20"/>
-      <c r="AK11" s="20" t="s">
-        <v>258</v>
-      </c>
+      <c r="AB11" s="24" t="s">
+        <v>270</v>
+      </c>
+      <c r="AC11" s="20">
+        <v>46294</v>
+      </c>
+      <c r="AK11" s="20"/>
     </row>
     <row r="12" spans="1:37">
       <c r="A12" s="11" t="s">
@@ -2476,14 +2569,19 @@
       <c r="Y12" s="20">
         <v>46268</v>
       </c>
+      <c r="Z12" s="20">
+        <v>46279</v>
+      </c>
       <c r="AA12" s="24">
         <v>46279</v>
       </c>
-      <c r="AB12" s="24"/>
-      <c r="AC12" s="20"/>
-      <c r="AK12" s="20" t="s">
-        <v>252</v>
-      </c>
+      <c r="AB12" s="24">
+        <v>46293</v>
+      </c>
+      <c r="AC12" s="20">
+        <v>46294</v>
+      </c>
+      <c r="AK12" s="20"/>
     </row>
     <row r="13" spans="1:37">
       <c r="A13" s="11" t="s">
@@ -2573,9 +2671,7 @@
       <c r="AC13" s="20">
         <v>46287</v>
       </c>
-      <c r="AK13" s="20" t="s">
-        <v>251</v>
-      </c>
+      <c r="AK13" s="20"/>
     </row>
     <row r="14" spans="1:37">
       <c r="A14" s="11" t="s">
@@ -2722,8 +2818,12 @@
       <c r="R15" s="20">
         <v>46275</v>
       </c>
-      <c r="S15" s="20"/>
-      <c r="T15" s="20"/>
+      <c r="S15" s="20">
+        <v>46275</v>
+      </c>
+      <c r="T15" s="20">
+        <v>46289</v>
+      </c>
       <c r="U15" s="20"/>
       <c r="V15" s="20"/>
       <c r="W15" s="20"/>
@@ -2746,7 +2846,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G16" s="19" t="s">
         <v>177</v>
@@ -2758,7 +2858,6 @@
         <v>46321</v>
       </c>
       <c r="J16" s="21"/>
-      <c r="K16" s="20"/>
       <c r="L16" s="20"/>
       <c r="M16" s="20"/>
       <c r="N16" s="20"/>
@@ -2766,7 +2865,6 @@
       <c r="P16" s="20"/>
       <c r="Q16" s="20"/>
       <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
     </row>
@@ -2787,7 +2885,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G17" s="19" t="s">
         <v>165</v>
@@ -2801,13 +2899,11 @@
       <c r="J17" s="21"/>
       <c r="K17" s="20"/>
       <c r="L17" s="20"/>
-      <c r="M17" s="20"/>
       <c r="N17" s="20"/>
       <c r="O17" s="20"/>
       <c r="P17" s="20"/>
       <c r="Q17" s="20"/>
       <c r="R17" s="20"/>
-      <c r="S17" s="20"/>
       <c r="T17" s="20"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20"/>
@@ -2828,10 +2924,10 @@
         <v>65</v>
       </c>
       <c r="E18" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>207</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>208</v>
       </c>
       <c r="G18" s="19" t="s">
         <v>178</v>
@@ -2847,7 +2943,6 @@
       <c r="L18" s="20"/>
       <c r="M18" s="20"/>
       <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
       <c r="P18" s="20"/>
       <c r="Q18" s="20"/>
       <c r="R18" s="20"/>
@@ -2869,10 +2964,10 @@
         <v>27</v>
       </c>
       <c r="E19" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="F19" s="19" t="s">
         <v>209</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>210</v>
       </c>
       <c r="G19" s="19" t="s">
         <v>179</v>
@@ -2890,9 +2985,6 @@
       <c r="N19" s="20"/>
       <c r="O19" s="20"/>
       <c r="P19" s="20"/>
-      <c r="Q19" s="20"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20"/>
       <c r="T19" s="20"/>
       <c r="U19" s="20"/>
       <c r="V19" s="20"/>
@@ -2916,7 +3008,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G20" s="19" t="s">
         <v>180</v>
@@ -2957,7 +3049,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G21" s="19" t="s">
         <v>181</v>
@@ -2972,13 +3064,6 @@
       <c r="K21" s="20"/>
       <c r="L21" s="20"/>
       <c r="M21" s="20"/>
-      <c r="N21" s="20"/>
-      <c r="O21" s="20"/>
-      <c r="P21" s="20"/>
-      <c r="Q21" s="20"/>
-      <c r="R21" s="20"/>
-      <c r="S21" s="20"/>
-      <c r="T21" s="20"/>
       <c r="U21" s="20"/>
       <c r="V21" s="20"/>
       <c r="W21" s="20"/>
@@ -3001,7 +3086,7 @@
         <v>15</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G22" s="19" t="s">
         <v>182</v>
@@ -3018,7 +3103,9 @@
       <c r="K22" s="20">
         <v>46287</v>
       </c>
-      <c r="L22" s="20"/>
+      <c r="L22" s="20">
+        <v>46289</v>
+      </c>
       <c r="M22" s="20"/>
       <c r="N22" s="20"/>
       <c r="O22" s="20"/>
@@ -3043,7 +3130,7 @@
         <v>14</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>74</v>
@@ -3087,10 +3174,10 @@
         <v>175</v>
       </c>
       <c r="E24" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="F24" s="19" t="s">
         <v>215</v>
-      </c>
-      <c r="F24" s="19" t="s">
-        <v>216</v>
       </c>
       <c r="G24" s="19" t="s">
         <v>184</v>
@@ -3106,9 +3193,6 @@
       <c r="L24" s="20"/>
       <c r="M24" s="20"/>
       <c r="N24" s="20"/>
-      <c r="O24" s="20"/>
-      <c r="P24" s="20"/>
-      <c r="Q24" s="20"/>
       <c r="R24" s="20"/>
       <c r="S24" s="20"/>
       <c r="T24" s="20"/>
@@ -3128,10 +3212,10 @@
         <v>13</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G25" s="19" t="s">
         <v>185</v>
@@ -3226,7 +3310,7 @@
         <v>3</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G27" s="19" t="s">
         <v>171</v>
@@ -3243,9 +3327,15 @@
       <c r="K27" s="20">
         <v>46287</v>
       </c>
-      <c r="L27" s="20"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="20"/>
+      <c r="L27" s="20">
+        <v>46289</v>
+      </c>
+      <c r="M27" s="20">
+        <v>46290</v>
+      </c>
+      <c r="N27" s="20">
+        <v>46295</v>
+      </c>
       <c r="O27" s="20"/>
       <c r="P27" s="20"/>
       <c r="Q27" s="20"/>
@@ -3271,10 +3361,10 @@
         <v>49</v>
       </c>
       <c r="E28" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="F28" s="19" t="s">
         <v>219</v>
-      </c>
-      <c r="F28" s="19" t="s">
-        <v>220</v>
       </c>
       <c r="G28" s="19" t="s">
         <v>186</v>
@@ -3315,7 +3405,7 @@
         <v>1</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G29" s="19" t="s">
         <v>187</v>
@@ -3356,10 +3446,10 @@
         <v>306</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G30" s="19" t="s">
         <v>188</v>
@@ -3400,7 +3490,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G31" s="19" t="s">
         <v>190</v>
@@ -3441,7 +3531,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G32" s="19" t="s">
         <v>189</v>
@@ -3482,10 +3572,10 @@
         <v>16</v>
       </c>
       <c r="E33" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="F33" s="19" t="s">
         <v>224</v>
-      </c>
-      <c r="F33" s="19" t="s">
-        <v>225</v>
       </c>
       <c r="G33" s="19" t="s">
         <v>191</v>
@@ -3505,8 +3595,12 @@
       <c r="L33" s="20">
         <v>46274</v>
       </c>
-      <c r="M33" s="20"/>
-      <c r="N33" s="20"/>
+      <c r="M33" s="20">
+        <v>46293</v>
+      </c>
+      <c r="N33" s="20">
+        <v>46295</v>
+      </c>
       <c r="O33" s="20"/>
       <c r="P33" s="20"/>
       <c r="Q33" s="20"/>
@@ -3529,13 +3623,13 @@
         <v>5</v>
       </c>
       <c r="D34" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="E34" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="F34" s="19" t="s">
         <v>227</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>228</v>
       </c>
       <c r="G34" s="19" t="s">
         <v>192</v>
@@ -3547,10 +3641,6 @@
         <v>46363</v>
       </c>
       <c r="J34" s="21"/>
-      <c r="K34" s="20"/>
-      <c r="L34" s="20"/>
-      <c r="M34" s="20"/>
-      <c r="N34" s="20"/>
       <c r="O34" s="20"/>
       <c r="P34" s="20"/>
       <c r="Q34" s="20"/>
@@ -3576,7 +3666,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G35" s="19" t="s">
         <v>171</v>
@@ -3590,8 +3680,6 @@
       <c r="J35" s="21"/>
       <c r="K35" s="20"/>
       <c r="L35" s="20"/>
-      <c r="M35" s="20"/>
-      <c r="N35" s="20"/>
       <c r="O35" s="20"/>
       <c r="P35" s="20"/>
       <c r="Q35" s="20"/>
@@ -3620,7 +3708,7 @@
         <v>4</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G36" s="19" t="s">
         <v>179</v>
@@ -3631,9 +3719,6 @@
       <c r="I36" s="21">
         <v>46363</v>
       </c>
-      <c r="J36" s="21"/>
-      <c r="K36" s="20"/>
-      <c r="L36" s="20"/>
       <c r="M36" s="20"/>
       <c r="N36" s="20"/>
       <c r="O36" s="20"/>
@@ -3655,13 +3740,13 @@
         <v>8</v>
       </c>
       <c r="D37" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="E37" s="11" t="s">
+      <c r="F37" s="19" t="s">
         <v>232</v>
-      </c>
-      <c r="F37" s="19" t="s">
-        <v>233</v>
       </c>
       <c r="G37" s="19" t="s">
         <v>193</v>
@@ -3672,9 +3757,6 @@
       <c r="I37" s="21">
         <v>46363</v>
       </c>
-      <c r="J37" s="21"/>
-      <c r="K37" s="20"/>
-      <c r="L37" s="20"/>
       <c r="M37" s="20"/>
       <c r="N37" s="20"/>
       <c r="O37" s="20"/>
@@ -3705,7 +3787,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G38" s="19" t="s">
         <v>171</v>
@@ -3722,9 +3804,15 @@
       <c r="K38" s="20">
         <v>46287</v>
       </c>
-      <c r="L38" s="20"/>
-      <c r="M38" s="20"/>
-      <c r="N38" s="20"/>
+      <c r="L38" s="20">
+        <v>46289</v>
+      </c>
+      <c r="M38" s="20">
+        <v>46290</v>
+      </c>
+      <c r="N38" s="20">
+        <v>46293</v>
+      </c>
       <c r="O38" s="20"/>
       <c r="P38" s="20"/>
       <c r="Q38" s="20"/>
@@ -3747,13 +3835,13 @@
         <v>14</v>
       </c>
       <c r="E39" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="F39" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="F39" s="19" t="s">
-        <v>236</v>
-      </c>
       <c r="G39" s="19" t="s">
-        <v>194</v>
+        <v>252</v>
       </c>
       <c r="H39" s="21">
         <v>46449</v>
@@ -3788,16 +3876,16 @@
         <v>1</v>
       </c>
       <c r="D40" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="E40" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="E40" s="11" t="s">
-        <v>238</v>
-      </c>
       <c r="F40" s="19" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H40" s="21">
         <v>46491</v>
@@ -3832,13 +3920,13 @@
         <v>284</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H41" s="21">
         <v>46491</v>
@@ -3879,10 +3967,10 @@
         <v>6</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H42" s="21">
         <v>46491</v>
@@ -3905,25 +3993,25 @@
     </row>
     <row r="43" spans="1:24">
       <c r="A43" s="11" t="s">
-        <v>144</v>
+        <v>251</v>
       </c>
       <c r="B43" t="s">
-        <v>145</v>
+        <v>253</v>
       </c>
       <c r="C43" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D43" s="11">
-        <v>270</v>
-      </c>
-      <c r="E43" s="11">
-        <v>2</v>
+        <v>167</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>255</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>198</v>
+        <v>254</v>
       </c>
       <c r="H43" s="21">
         <v>46491</v>
@@ -3949,25 +4037,25 @@
     </row>
     <row r="44" spans="1:24">
       <c r="A44" s="11" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C44" s="11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D44" s="11">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="E44" s="11">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>240</v>
+        <v>211</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H44" s="21">
         <v>46491</v>
@@ -3987,28 +4075,31 @@
       <c r="S44" s="20"/>
       <c r="T44" s="20"/>
       <c r="U44" s="20"/>
+      <c r="V44" s="20"/>
+      <c r="W44" s="20"/>
+      <c r="X44" s="20"/>
     </row>
     <row r="45" spans="1:24">
       <c r="A45" s="11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B45" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C45" s="11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D45" s="11">
-        <v>365</v>
+        <v>9</v>
       </c>
       <c r="E45" s="11">
         <v>12</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>76</v>
+        <v>239</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H45" s="21">
         <v>46491</v>
@@ -4028,31 +4119,28 @@
       <c r="S45" s="20"/>
       <c r="T45" s="20"/>
       <c r="U45" s="20"/>
-      <c r="V45" s="20"/>
-      <c r="W45" s="20"/>
-      <c r="X45" s="20"/>
     </row>
     <row r="46" spans="1:24">
       <c r="A46" s="11" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B46" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C46" s="11">
-        <v>7</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="E46" s="11" t="s">
-        <v>242</v>
+        <v>6</v>
+      </c>
+      <c r="D46" s="11">
+        <v>365</v>
+      </c>
+      <c r="E46" s="11">
+        <v>12</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>243</v>
+        <v>76</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H46" s="21">
         <v>46491</v>
@@ -4072,28 +4160,31 @@
       <c r="S46" s="20"/>
       <c r="T46" s="20"/>
       <c r="U46" s="20"/>
+      <c r="V46" s="20"/>
+      <c r="W46" s="20"/>
+      <c r="X46" s="20"/>
     </row>
     <row r="47" spans="1:24">
       <c r="A47" s="11" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C47" s="11">
-        <v>9</v>
-      </c>
-      <c r="D47" s="11">
-        <v>65</v>
+        <v>7</v>
+      </c>
+      <c r="D47" s="11" t="s">
+        <v>240</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="H47" s="21">
         <v>46491</v>
@@ -4113,31 +4204,28 @@
       <c r="S47" s="20"/>
       <c r="T47" s="20"/>
       <c r="U47" s="20"/>
-      <c r="V47" s="20"/>
-      <c r="W47" s="20"/>
-      <c r="X47" s="20"/>
     </row>
     <row r="48" spans="1:24">
       <c r="A48" s="11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B48" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C48" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D48" s="11">
-        <v>90</v>
-      </c>
-      <c r="E48" s="11">
-        <v>6</v>
+        <v>65</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>243</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>202</v>
+        <v>171</v>
       </c>
       <c r="H48" s="21">
         <v>46491</v>
@@ -4157,34 +4245,37 @@
       <c r="S48" s="20"/>
       <c r="T48" s="20"/>
       <c r="U48" s="20"/>
+      <c r="V48" s="20"/>
+      <c r="W48" s="20"/>
+      <c r="X48" s="20"/>
     </row>
     <row r="49" spans="1:24">
       <c r="A49" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B49" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C49" s="11">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D49" s="11">
-        <v>385</v>
+        <v>90</v>
       </c>
       <c r="E49" s="11">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>72</v>
+        <v>245</v>
       </c>
       <c r="G49" s="19" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H49" s="21">
-        <v>46526</v>
+        <v>46491</v>
       </c>
       <c r="I49" s="21">
-        <v>46440</v>
+        <v>46398</v>
       </c>
       <c r="J49" s="21"/>
       <c r="K49" s="20"/>
@@ -4198,28 +4289,25 @@
       <c r="S49" s="20"/>
       <c r="T49" s="20"/>
       <c r="U49" s="20"/>
-      <c r="V49" s="20"/>
-      <c r="W49" s="20"/>
-      <c r="X49" s="20"/>
     </row>
     <row r="50" spans="1:24">
       <c r="A50" s="11" t="s">
-        <v>158</v>
+        <v>256</v>
       </c>
       <c r="B50" t="s">
-        <v>159</v>
+        <v>261</v>
       </c>
       <c r="C50" s="11">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D50" s="11">
-        <v>65</v>
-      </c>
-      <c r="E50" s="11" t="s">
-        <v>219</v>
+        <v>52</v>
+      </c>
+      <c r="E50" s="11">
+        <v>0</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>247</v>
+        <v>267</v>
       </c>
       <c r="G50" s="19" t="s">
         <v>177</v>
@@ -4245,25 +4333,25 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" s="11" t="s">
-        <v>160</v>
+        <v>257</v>
       </c>
       <c r="B51" t="s">
-        <v>161</v>
+        <v>262</v>
       </c>
       <c r="C51" s="11">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D51" s="11">
-        <v>49</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>209</v>
+        <v>71</v>
+      </c>
+      <c r="E51" s="11">
+        <v>4</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>248</v>
+        <v>268</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>204</v>
+        <v>175</v>
       </c>
       <c r="H51" s="21">
         <v>46526</v>
@@ -4288,26 +4376,26 @@
       <c r="X51" s="20"/>
     </row>
     <row r="52" spans="1:24">
-      <c r="A52" s="23" t="s">
-        <v>250</v>
+      <c r="A52" s="11" t="s">
+        <v>156</v>
       </c>
       <c r="B52" t="s">
-        <v>249</v>
+        <v>157</v>
       </c>
       <c r="C52" s="11">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D52" s="11">
-        <v>412</v>
+        <v>385</v>
       </c>
       <c r="E52" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>218</v>
+        <v>72</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>171</v>
+        <v>202</v>
       </c>
       <c r="H52" s="21">
         <v>46526</v>
@@ -4327,6 +4415,264 @@
       <c r="S52" s="20"/>
       <c r="T52" s="20"/>
       <c r="U52" s="20"/>
+      <c r="V52" s="20"/>
+      <c r="W52" s="20"/>
+      <c r="X52" s="20"/>
+    </row>
+    <row r="53" spans="1:24">
+      <c r="A53" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="B53" t="s">
+        <v>263</v>
+      </c>
+      <c r="C53" s="11">
+        <v>6</v>
+      </c>
+      <c r="D53" s="11">
+        <v>128</v>
+      </c>
+      <c r="E53" s="11">
+        <v>10</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>269</v>
+      </c>
+      <c r="G53" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H53" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I53" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J53" s="21"/>
+      <c r="K53" s="20"/>
+      <c r="L53" s="20"/>
+      <c r="M53" s="20"/>
+      <c r="N53" s="20"/>
+      <c r="O53" s="20"/>
+      <c r="P53" s="20"/>
+      <c r="Q53" s="20"/>
+      <c r="R53" s="20"/>
+      <c r="S53" s="20"/>
+      <c r="T53" s="20"/>
+      <c r="U53" s="20"/>
+    </row>
+    <row r="54" spans="1:24">
+      <c r="A54" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="B54" t="s">
+        <v>264</v>
+      </c>
+      <c r="C54" s="11">
+        <v>7</v>
+      </c>
+      <c r="D54" s="11">
+        <v>53</v>
+      </c>
+      <c r="E54" s="11">
+        <v>1</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G54" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="H54" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I54" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J54" s="21"/>
+      <c r="K54" s="20"/>
+      <c r="L54" s="20"/>
+      <c r="M54" s="20"/>
+      <c r="N54" s="20"/>
+      <c r="O54" s="20"/>
+      <c r="P54" s="20"/>
+      <c r="Q54" s="20"/>
+      <c r="R54" s="20"/>
+      <c r="S54" s="20"/>
+      <c r="T54" s="20"/>
+      <c r="U54" s="20"/>
+    </row>
+    <row r="55" spans="1:24">
+      <c r="A55" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="B55" t="s">
+        <v>265</v>
+      </c>
+      <c r="C55" s="11">
+        <v>9</v>
+      </c>
+      <c r="D55" s="11">
+        <v>71</v>
+      </c>
+      <c r="E55" s="11">
+        <v>19</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="G55" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="H55" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I55" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J55" s="21"/>
+      <c r="K55" s="20"/>
+      <c r="L55" s="20"/>
+      <c r="M55" s="20"/>
+      <c r="N55" s="20"/>
+      <c r="O55" s="20"/>
+      <c r="P55" s="20"/>
+      <c r="Q55" s="20"/>
+      <c r="R55" s="20"/>
+      <c r="S55" s="20"/>
+      <c r="T55" s="20"/>
+      <c r="U55" s="20"/>
+      <c r="V55" s="20"/>
+      <c r="W55" s="20"/>
+      <c r="X55" s="20"/>
+    </row>
+    <row r="56" spans="1:24">
+      <c r="A56" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="B56" t="s">
+        <v>159</v>
+      </c>
+      <c r="C56" s="11">
+        <v>9</v>
+      </c>
+      <c r="D56" s="11">
+        <v>65</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="F56" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="G56" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="H56" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I56" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J56" s="21"/>
+      <c r="K56" s="20"/>
+      <c r="L56" s="20"/>
+      <c r="M56" s="20"/>
+      <c r="N56" s="20"/>
+      <c r="O56" s="20"/>
+      <c r="P56" s="20"/>
+      <c r="Q56" s="20"/>
+      <c r="R56" s="20"/>
+      <c r="S56" s="20"/>
+      <c r="T56" s="20"/>
+      <c r="U56" s="20"/>
+      <c r="V56" s="20"/>
+      <c r="W56" s="20"/>
+      <c r="X56" s="20"/>
+    </row>
+    <row r="57" spans="1:24">
+      <c r="A57" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B57" t="s">
+        <v>161</v>
+      </c>
+      <c r="C57" s="11">
+        <v>10</v>
+      </c>
+      <c r="D57" s="11">
+        <v>49</v>
+      </c>
+      <c r="E57" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="F57" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="G57" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="H57" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I57" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J57" s="21"/>
+      <c r="K57" s="20"/>
+      <c r="L57" s="20"/>
+      <c r="M57" s="20"/>
+      <c r="N57" s="20"/>
+      <c r="O57" s="20"/>
+      <c r="P57" s="20"/>
+      <c r="Q57" s="20"/>
+      <c r="R57" s="20"/>
+      <c r="S57" s="20"/>
+      <c r="T57" s="20"/>
+      <c r="U57" s="20"/>
+      <c r="V57" s="20"/>
+      <c r="W57" s="20"/>
+      <c r="X57" s="20"/>
+    </row>
+    <row r="58" spans="1:24">
+      <c r="A58" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="B58" t="s">
+        <v>248</v>
+      </c>
+      <c r="C58" s="11">
+        <v>9</v>
+      </c>
+      <c r="D58" s="11">
+        <v>412</v>
+      </c>
+      <c r="E58" s="11">
+        <v>1</v>
+      </c>
+      <c r="F58" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="G58" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="H58" s="21">
+        <v>46526</v>
+      </c>
+      <c r="I58" s="21">
+        <v>46440</v>
+      </c>
+      <c r="J58" s="21"/>
+      <c r="K58" s="20"/>
+      <c r="L58" s="20"/>
+      <c r="M58" s="20"/>
+      <c r="N58" s="20"/>
+      <c r="O58" s="20"/>
+      <c r="P58" s="20"/>
+      <c r="Q58" s="20"/>
+      <c r="R58" s="20"/>
+      <c r="S58" s="20"/>
+      <c r="T58" s="20"/>
+      <c r="U58" s="20"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
Major Update on PPP 2027 on 10.14.26
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{96CAE750-3891-4C13-A1A6-B95BF8A82FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED35B639-C39C-4866-90E0-42B1C21E1D9F}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{908BCBEC-4003-4C53-A1F3-237188509867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{147AD658-2F46-437E-96AF-C7EB2A4CE2FE}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="270">
   <si>
     <t>1st Review</t>
   </si>
@@ -135,24 +135,6 @@
     <t>CCD Corrections</t>
   </si>
   <si>
-    <t>Returned to SB</t>
-  </si>
-  <si>
-    <t>Returned to CCD</t>
-  </si>
-  <si>
-    <t>Addendum 1 Sent to Dist</t>
-  </si>
-  <si>
-    <t>Addendum 1 to SB</t>
-  </si>
-  <si>
-    <t>Additional comments to District</t>
-  </si>
-  <si>
-    <t>Sent to SB</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
@@ -171,9 +153,6 @@
     <t>Turnaround Days (Optional)</t>
   </si>
   <si>
-    <t>Workflow complete</t>
-  </si>
-  <si>
     <t>A10059</t>
   </si>
   <si>
@@ -786,9 +765,6 @@
     <t>090735</t>
   </si>
   <si>
-    <t>9/112026</t>
-  </si>
-  <si>
     <t>A20046</t>
   </si>
   <si>
@@ -849,7 +825,25 @@
     <t>9/258/2026</t>
   </si>
   <si>
-    <t>Waiting on correction from District</t>
+    <t>District is waiting on Mix Design from Materials</t>
+  </si>
+  <si>
+    <t>Emailed district with the Reminder for October 26 Submission</t>
+  </si>
+  <si>
+    <t>Emailed Micah asking if it is ready for 2nd review @10.13.26</t>
+  </si>
+  <si>
+    <t>Emailed Bryce asking if it is ready for 3rd review @10.13.26</t>
+  </si>
+  <si>
+    <t>Emailed to Sharon for 3rd Review</t>
+  </si>
+  <si>
+    <t>Emailed Bryce asking if it is ready for 3rd review @10.14.26</t>
+  </si>
+  <si>
+    <t>Send for DE Signature</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1008,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1075,72 +1069,18 @@
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2A31118A-900B-4722-A90B-8152F5F4035D}"/>
   </cellStyles>
-  <dxfs count="14">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="8">
     <dxf>
       <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1205,24 +1145,20 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PPPProjectsTable" displayName="PPPProjectsTable" ref="A1:AK58" totalsRowShown="0">
-  <autoFilter ref="A1:AK58" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="37">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Job Number" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PPPProjectsTable" displayName="PPPProjectsTable" ref="A1:AD58" totalsRowShown="0">
+  <autoFilter ref="A1:AD58" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="30">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Job Number" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Project Description"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="District" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Route" dataDxfId="11"/>
-    <tableColumn id="36" xr3:uid="{B65E3A66-8F4F-4C7A-8EAC-7D6C80DA624C}" name="Section" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="County" dataDxfId="9"/>
-    <tableColumn id="37" xr3:uid="{91677106-A41F-4D5F-A2D6-7604E00D01E2}" name="Scope" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Letting Date" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="District" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Route" dataDxfId="5"/>
+    <tableColumn id="36" xr3:uid="{B65E3A66-8F4F-4C7A-8EAC-7D6C80DA624C}" name="Section" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="County" dataDxfId="3"/>
+    <tableColumn id="37" xr3:uid="{91677106-A41F-4D5F-A2D6-7604E00D01E2}" name="Scope" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Letting Date" dataDxfId="1"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Due to PM"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="1st Review Sent to SB" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="1st Review Sent to SB" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="1st Review Returned from SB"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="1st Review Sent to District"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="1st Review Returned from District"/>
@@ -1242,13 +1178,6 @@
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Requested Title Sheet"/>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Received Signed Plans"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Sent to CCD"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="CCD Corrections"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Returned to SB"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Returned to CCD"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Addendum 1 Sent to Dist"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Addendum 1 to SB"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Additional comments to District"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Sent to SB"/>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1256,8 +1185,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="StageReferenceTable" displayName="StageReferenceTable" ref="A1:E28" totalsRowShown="0">
-  <autoFilter ref="A1:E28" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="StageReferenceTable" displayName="StageReferenceTable" ref="A1:E21" totalsRowShown="0">
+  <autoFilter ref="A1:E21" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Sequence"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Review Phase"/>
@@ -1464,7 +1393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AK58"/>
+  <dimension ref="A1:AD58"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1477,11 +1406,11 @@
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="18" style="11" customWidth="1"/>
     <col min="11" max="25" width="18" customWidth="1"/>
-    <col min="26" max="36" width="20" customWidth="1"/>
-    <col min="37" max="37" width="41.796875" customWidth="1"/>
+    <col min="26" max="29" width="20" customWidth="1"/>
+    <col min="30" max="30" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" ht="52.05" customHeight="1">
+    <row r="1" spans="1:30" ht="52.05" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -1495,13 +1424,13 @@
         <v>8</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>10</v>
@@ -1569,37 +1498,16 @@
       <c r="AC1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="AD1" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE1" s="8" t="s">
+      <c r="AD1" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="AF1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK1" s="9" t="s">
+    </row>
+    <row r="2" spans="1:30">
+      <c r="A2" s="11" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:37">
-      <c r="A2" s="11" t="s">
-        <v>46</v>
-      </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C2" s="11">
         <v>1</v>
@@ -1611,10 +1519,10 @@
         <v>1</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="H2" s="21">
         <v>46330</v>
@@ -1673,8 +1581,8 @@
       <c r="Z2" s="20">
         <v>46276</v>
       </c>
-      <c r="AA2" s="24" t="s">
-        <v>250</v>
+      <c r="AA2" s="24">
+        <v>46276</v>
       </c>
       <c r="AB2" s="24">
         <v>46288</v>
@@ -1682,14 +1590,14 @@
       <c r="AC2" s="20">
         <v>46288</v>
       </c>
-      <c r="AK2" s="20"/>
-    </row>
-    <row r="3" spans="1:37">
+      <c r="AD2" s="20"/>
+    </row>
+    <row r="3" spans="1:30">
       <c r="A3" s="11" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C3" s="11">
         <v>2</v>
@@ -1701,10 +1609,10 @@
         <v>6</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="H3" s="21">
         <v>46330</v>
@@ -1769,17 +1677,17 @@
       <c r="AB3" s="24">
         <v>46286</v>
       </c>
-      <c r="AC3" s="20"/>
-      <c r="AK3" s="20" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37">
+      <c r="AC3" s="20">
+        <v>46309</v>
+      </c>
+      <c r="AD3" s="20"/>
+    </row>
+    <row r="4" spans="1:30">
       <c r="A4" s="11" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C4" s="11">
         <v>3</v>
@@ -1788,13 +1696,13 @@
         <v>73</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="H4" s="21">
         <v>46330</v>
@@ -1863,12 +1771,12 @@
         <v>46275</v>
       </c>
     </row>
-    <row r="5" spans="1:37">
+    <row r="5" spans="1:30">
       <c r="A5" s="11" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C5" s="11">
         <v>4</v>
@@ -1880,10 +1788,10 @@
         <v>1</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="H5" s="21">
         <v>46330</v>
@@ -1951,14 +1859,14 @@
       <c r="AC5" s="20">
         <v>46282</v>
       </c>
-      <c r="AK5" s="25"/>
-    </row>
-    <row r="6" spans="1:37">
+      <c r="AD5" s="25"/>
+    </row>
+    <row r="6" spans="1:30">
       <c r="A6" s="11" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C6" s="11">
         <v>5</v>
@@ -1970,10 +1878,10 @@
         <v>15</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="H6" s="21">
         <v>46330</v>
@@ -2041,14 +1949,14 @@
       <c r="AC6" s="20">
         <v>46287</v>
       </c>
-      <c r="AK6" s="20"/>
-    </row>
-    <row r="7" spans="1:37">
+      <c r="AD6" s="20"/>
+    </row>
+    <row r="7" spans="1:30">
       <c r="A7" s="11" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C7" s="11">
         <v>5</v>
@@ -2060,10 +1968,10 @@
         <v>8</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="H7" s="21">
         <v>46330</v>
@@ -2131,14 +2039,14 @@
       <c r="AC7" s="20">
         <v>46287</v>
       </c>
-      <c r="AK7" s="20"/>
-    </row>
-    <row r="8" spans="1:37">
+      <c r="AD7" s="20"/>
+    </row>
+    <row r="8" spans="1:30">
       <c r="A8" s="11" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C8" s="11">
         <v>6</v>
@@ -2150,10 +2058,10 @@
         <v>2</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="H8" s="21">
         <v>46330</v>
@@ -2221,14 +2129,14 @@
       <c r="AC8" s="20">
         <v>46282</v>
       </c>
-      <c r="AK8" s="20"/>
-    </row>
-    <row r="9" spans="1:37">
+      <c r="AD8" s="20"/>
+    </row>
+    <row r="9" spans="1:30">
       <c r="A9" s="11" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C9" s="11">
         <v>7</v>
@@ -2240,10 +2148,10 @@
         <v>3</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H9" s="21">
         <v>46330</v>
@@ -2311,14 +2219,14 @@
       <c r="AC9" s="20">
         <v>46279</v>
       </c>
-      <c r="AK9" s="20"/>
-    </row>
-    <row r="10" spans="1:37">
+      <c r="AD9" s="20"/>
+    </row>
+    <row r="10" spans="1:30">
       <c r="A10" s="11" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C10" s="11">
         <v>7</v>
@@ -2330,10 +2238,10 @@
         <v>0</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G10" s="19" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="H10" s="21">
         <v>46330</v>
@@ -2401,14 +2309,14 @@
       <c r="AC10" s="20">
         <v>46288</v>
       </c>
-      <c r="AK10" s="20"/>
-    </row>
-    <row r="11" spans="1:37">
+      <c r="AD10" s="20"/>
+    </row>
+    <row r="11" spans="1:30">
       <c r="A11" s="11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C11" s="11">
         <v>8</v>
@@ -2420,10 +2328,10 @@
         <v>8</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="H11" s="21">
         <v>46330</v>
@@ -2486,19 +2394,19 @@
         <v>46286</v>
       </c>
       <c r="AB11" s="24" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="AC11" s="20">
         <v>46294</v>
       </c>
-      <c r="AK11" s="20"/>
-    </row>
-    <row r="12" spans="1:37">
+      <c r="AD11" s="20"/>
+    </row>
+    <row r="12" spans="1:30">
       <c r="A12" s="11" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C12" s="11">
         <v>9</v>
@@ -2510,10 +2418,10 @@
         <v>1</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H12" s="21">
         <v>46330</v>
@@ -2581,14 +2489,14 @@
       <c r="AC12" s="20">
         <v>46294</v>
       </c>
-      <c r="AK12" s="20"/>
-    </row>
-    <row r="13" spans="1:37">
+      <c r="AD12" s="20"/>
+    </row>
+    <row r="13" spans="1:30">
       <c r="A13" s="11" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C13" s="11">
         <v>9</v>
@@ -2597,13 +2505,13 @@
         <v>412</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="H13" s="21">
         <v>46330</v>
@@ -2671,14 +2579,14 @@
       <c r="AC13" s="20">
         <v>46287</v>
       </c>
-      <c r="AK13" s="20"/>
-    </row>
-    <row r="14" spans="1:37">
+      <c r="AD13" s="20"/>
+    </row>
+    <row r="14" spans="1:30">
       <c r="A14" s="11" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C14" s="11">
         <v>10</v>
@@ -2690,10 +2598,10 @@
         <v>4</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="H14" s="21">
         <v>46330</v>
@@ -2761,14 +2669,14 @@
       <c r="AC14" s="20">
         <v>46279</v>
       </c>
-      <c r="AK14" s="20"/>
-    </row>
-    <row r="15" spans="1:37">
+      <c r="AD14" s="20"/>
+    </row>
+    <row r="15" spans="1:30">
       <c r="A15" s="11" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C15" s="11">
         <v>1</v>
@@ -2780,10 +2688,10 @@
         <v>10</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="H15" s="21">
         <v>46407</v>
@@ -2824,17 +2732,37 @@
       <c r="T15" s="20">
         <v>46289</v>
       </c>
-      <c r="U15" s="20"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="20"/>
-    </row>
-    <row r="16" spans="1:37">
+      <c r="U15" s="20">
+        <v>46300</v>
+      </c>
+      <c r="V15" s="20">
+        <v>46300</v>
+      </c>
+      <c r="W15" s="20">
+        <v>46301</v>
+      </c>
+      <c r="X15" s="20">
+        <v>46301</v>
+      </c>
+      <c r="Y15" s="20">
+        <v>46303</v>
+      </c>
+      <c r="Z15" s="20">
+        <v>46308</v>
+      </c>
+      <c r="AA15" s="24">
+        <v>46308</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30">
       <c r="A16" s="11" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C16" s="11">
         <v>1</v>
@@ -2846,10 +2774,10 @@
         <v>1</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="G16" s="19" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="H16" s="21">
         <v>46407</v>
@@ -2867,13 +2795,16 @@
       <c r="R16" s="20"/>
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
-    </row>
-    <row r="17" spans="1:24">
+      <c r="AD16" s="20" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="17" spans="1:30">
       <c r="A17" s="11" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C17" s="11">
         <v>2</v>
@@ -2885,10 +2816,10 @@
         <v>2</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="H17" s="21">
         <v>46407</v>
@@ -2909,13 +2840,16 @@
       <c r="V17" s="20"/>
       <c r="W17" s="20"/>
       <c r="X17" s="20"/>
-    </row>
-    <row r="18" spans="1:24">
+      <c r="AD17" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:30">
       <c r="A18" s="11" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C18" s="11">
         <v>2</v>
@@ -2924,13 +2858,13 @@
         <v>65</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="H18" s="21">
         <v>46407</v>
@@ -2938,24 +2872,29 @@
       <c r="I18" s="21">
         <v>46321</v>
       </c>
-      <c r="J18" s="21"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="P18" s="20"/>
-      <c r="Q18" s="20"/>
-      <c r="R18" s="20"/>
-      <c r="S18" s="20"/>
-      <c r="T18" s="20"/>
-      <c r="U18" s="20"/>
-    </row>
-    <row r="19" spans="1:24">
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="26"/>
+      <c r="Q18" s="26"/>
+      <c r="R18" s="26"/>
+      <c r="S18" s="26"/>
+      <c r="T18" s="26"/>
+      <c r="U18" s="26"/>
+      <c r="V18" s="27"/>
+      <c r="AD18" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19" spans="1:30">
       <c r="A19" s="11" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C19" s="11">
         <v>3</v>
@@ -2964,13 +2903,13 @@
         <v>27</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H19" s="21">
         <v>46407</v>
@@ -2978,25 +2917,31 @@
       <c r="I19" s="21">
         <v>46321</v>
       </c>
-      <c r="J19" s="21"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="T19" s="20"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="27"/>
+      <c r="R19" s="27"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="26"/>
+      <c r="U19" s="26"/>
+      <c r="V19" s="26"/>
       <c r="W19" s="20"/>
       <c r="X19" s="20"/>
-    </row>
-    <row r="20" spans="1:24">
+      <c r="AD19" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="20" spans="1:30">
       <c r="A20" s="11" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B20" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C20" s="11">
         <v>3</v>
@@ -3008,10 +2953,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="H20" s="21">
         <v>46407</v>
@@ -3019,25 +2964,29 @@
       <c r="I20" s="21">
         <v>46321</v>
       </c>
-      <c r="J20" s="21"/>
-      <c r="K20" s="20"/>
-      <c r="L20" s="20"/>
-      <c r="M20" s="20"/>
-      <c r="N20" s="20"/>
-      <c r="O20" s="20"/>
-      <c r="P20" s="20"/>
-      <c r="Q20" s="20"/>
-      <c r="R20" s="20"/>
-      <c r="S20" s="20"/>
-      <c r="T20" s="20"/>
-      <c r="U20" s="20"/>
-    </row>
-    <row r="21" spans="1:24">
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="26"/>
+      <c r="R20" s="26"/>
+      <c r="S20" s="26"/>
+      <c r="T20" s="26"/>
+      <c r="U20" s="26"/>
+      <c r="V20" s="27"/>
+      <c r="AD20" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="21" spans="1:30">
       <c r="A21" s="11" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C21" s="11">
         <v>4</v>
@@ -3049,10 +2998,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="H21" s="21">
         <v>46407</v>
@@ -3060,21 +3009,31 @@
       <c r="I21" s="21">
         <v>46321</v>
       </c>
-      <c r="J21" s="21"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="20"/>
-      <c r="M21" s="20"/>
-      <c r="U21" s="20"/>
-      <c r="V21" s="20"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="27"/>
+      <c r="U21" s="26"/>
+      <c r="V21" s="26"/>
       <c r="W21" s="20"/>
       <c r="X21" s="20"/>
-    </row>
-    <row r="22" spans="1:24">
+      <c r="AD21" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="1:30">
       <c r="A22" s="11" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C22" s="11">
         <v>5</v>
@@ -3086,10 +3045,10 @@
         <v>15</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="H22" s="21">
         <v>46407</v>
@@ -3097,31 +3056,35 @@
       <c r="I22" s="21">
         <v>46321</v>
       </c>
-      <c r="J22" s="21">
+      <c r="J22" s="26">
         <v>46283</v>
       </c>
-      <c r="K22" s="20">
+      <c r="K22" s="26">
         <v>46287</v>
       </c>
-      <c r="L22" s="20">
+      <c r="L22" s="26">
         <v>46289</v>
       </c>
-      <c r="M22" s="20"/>
-      <c r="N22" s="20"/>
-      <c r="O22" s="20"/>
-      <c r="P22" s="20"/>
-      <c r="Q22" s="20"/>
-      <c r="R22" s="20"/>
-      <c r="S22" s="20"/>
-      <c r="T22" s="20"/>
-      <c r="U22" s="20"/>
-    </row>
-    <row r="23" spans="1:24">
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
+      <c r="Q22" s="26"/>
+      <c r="R22" s="26"/>
+      <c r="S22" s="26"/>
+      <c r="T22" s="26"/>
+      <c r="U22" s="26"/>
+      <c r="V22" s="27"/>
+      <c r="AD22" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="23" spans="1:30">
       <c r="A23" s="11" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B23" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C23" s="11">
         <v>5</v>
@@ -3130,13 +3093,13 @@
         <v>14</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="H23" s="21">
         <v>46407</v>
@@ -3144,28 +3107,31 @@
       <c r="I23" s="21">
         <v>46321</v>
       </c>
-      <c r="J23" s="21"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
-      <c r="N23" s="20"/>
-      <c r="O23" s="20"/>
-      <c r="P23" s="20"/>
-      <c r="Q23" s="20"/>
-      <c r="R23" s="20"/>
-      <c r="S23" s="20"/>
-      <c r="T23" s="20"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="20"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="26"/>
+      <c r="L23" s="26"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="26"/>
+      <c r="O23" s="26"/>
+      <c r="P23" s="26"/>
+      <c r="Q23" s="26"/>
+      <c r="R23" s="26"/>
+      <c r="S23" s="26"/>
+      <c r="T23" s="26"/>
+      <c r="U23" s="26"/>
+      <c r="V23" s="26"/>
       <c r="W23" s="20"/>
       <c r="X23" s="20"/>
-    </row>
-    <row r="24" spans="1:24">
+      <c r="AD23" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="24" spans="1:30">
       <c r="A24" s="11" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B24" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C24" s="11">
         <v>5</v>
@@ -3174,13 +3140,13 @@
         <v>175</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="H24" s="21">
         <v>46407</v>
@@ -3188,22 +3154,29 @@
       <c r="I24" s="21">
         <v>46321</v>
       </c>
-      <c r="J24" s="21"/>
-      <c r="K24" s="20"/>
-      <c r="L24" s="20"/>
-      <c r="M24" s="20"/>
-      <c r="N24" s="20"/>
-      <c r="R24" s="20"/>
-      <c r="S24" s="20"/>
-      <c r="T24" s="20"/>
-      <c r="U24" s="20"/>
-    </row>
-    <row r="25" spans="1:24">
+      <c r="J24" s="26"/>
+      <c r="K24" s="26"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="26"/>
+      <c r="N24" s="26"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="26"/>
+      <c r="S24" s="26"/>
+      <c r="T24" s="26"/>
+      <c r="U24" s="26"/>
+      <c r="V24" s="27"/>
+      <c r="AD24" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="25" spans="1:30">
       <c r="A25" s="11" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="C25" s="11">
         <v>6</v>
@@ -3212,13 +3185,13 @@
         <v>13</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="H25" s="21">
         <v>46407</v>
@@ -3226,28 +3199,31 @@
       <c r="I25" s="21">
         <v>46321</v>
       </c>
-      <c r="J25" s="21"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
-      <c r="M25" s="20"/>
-      <c r="N25" s="20"/>
-      <c r="O25" s="20"/>
-      <c r="P25" s="20"/>
-      <c r="Q25" s="20"/>
-      <c r="R25" s="20"/>
-      <c r="S25" s="20"/>
-      <c r="T25" s="20"/>
-      <c r="U25" s="20"/>
-      <c r="V25" s="20"/>
+      <c r="J25" s="26"/>
+      <c r="K25" s="26"/>
+      <c r="L25" s="26"/>
+      <c r="M25" s="26"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="26"/>
+      <c r="P25" s="26"/>
+      <c r="Q25" s="26"/>
+      <c r="R25" s="26"/>
+      <c r="S25" s="26"/>
+      <c r="T25" s="26"/>
+      <c r="U25" s="26"/>
+      <c r="V25" s="26"/>
       <c r="W25" s="20"/>
       <c r="X25" s="20"/>
-    </row>
-    <row r="26" spans="1:24">
+      <c r="AD25" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:30">
       <c r="A26" s="11" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C26" s="11">
         <v>7</v>
@@ -3259,10 +3235,10 @@
         <v>5</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H26" s="21">
         <v>46407</v>
@@ -3270,35 +3246,47 @@
       <c r="I26" s="21">
         <v>46321</v>
       </c>
-      <c r="J26" s="21">
+      <c r="J26" s="26">
         <v>46265</v>
       </c>
-      <c r="K26" s="20">
+      <c r="K26" s="26">
         <v>46270</v>
       </c>
-      <c r="L26" s="20">
+      <c r="L26" s="26">
         <v>46274</v>
       </c>
-      <c r="M26" s="20">
+      <c r="M26" s="26">
         <v>46275</v>
       </c>
-      <c r="N26" s="20">
+      <c r="N26" s="26">
         <v>46275</v>
       </c>
-      <c r="O26" s="20"/>
-      <c r="P26" s="20"/>
-      <c r="Q26" s="20"/>
-      <c r="R26" s="20"/>
-      <c r="S26" s="20"/>
-      <c r="T26" s="20"/>
-      <c r="U26" s="20"/>
-    </row>
-    <row r="27" spans="1:24">
+      <c r="O26" s="26">
+        <v>46275</v>
+      </c>
+      <c r="P26" s="26">
+        <v>46308</v>
+      </c>
+      <c r="Q26" s="26">
+        <v>46308</v>
+      </c>
+      <c r="R26" s="26">
+        <v>46308</v>
+      </c>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="26"/>
+      <c r="V26" s="27"/>
+      <c r="AD26" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="27" spans="1:30">
       <c r="A27" s="11" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B27" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C27" s="11">
         <v>9</v>
@@ -3310,10 +3298,10 @@
         <v>3</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H27" s="21">
         <v>46407</v>
@@ -3321,38 +3309,45 @@
       <c r="I27" s="21">
         <v>46321</v>
       </c>
-      <c r="J27" s="21">
+      <c r="J27" s="26">
         <v>46281</v>
       </c>
-      <c r="K27" s="20">
+      <c r="K27" s="26">
         <v>46287</v>
       </c>
-      <c r="L27" s="20">
+      <c r="L27" s="26">
         <v>46289</v>
       </c>
-      <c r="M27" s="20">
+      <c r="M27" s="26">
         <v>46290</v>
       </c>
-      <c r="N27" s="20">
+      <c r="N27" s="26">
         <v>46295</v>
       </c>
-      <c r="O27" s="20"/>
-      <c r="P27" s="20"/>
-      <c r="Q27" s="20"/>
-      <c r="R27" s="20"/>
-      <c r="S27" s="20"/>
-      <c r="T27" s="20"/>
-      <c r="U27" s="20"/>
-      <c r="V27" s="20"/>
+      <c r="O27" s="26">
+        <v>46295</v>
+      </c>
+      <c r="P27" s="26">
+        <v>46295</v>
+      </c>
+      <c r="Q27" s="26"/>
+      <c r="R27" s="26"/>
+      <c r="S27" s="26"/>
+      <c r="T27" s="26"/>
+      <c r="U27" s="26"/>
+      <c r="V27" s="26"/>
       <c r="W27" s="20"/>
       <c r="X27" s="20"/>
-    </row>
-    <row r="28" spans="1:24">
+      <c r="AD27" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="28" spans="1:30">
       <c r="A28" s="11" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="C28" s="11">
         <v>10</v>
@@ -3361,13 +3356,13 @@
         <v>49</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="H28" s="21">
         <v>46407</v>
@@ -3375,25 +3370,29 @@
       <c r="I28" s="21">
         <v>46321</v>
       </c>
-      <c r="J28" s="21"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20"/>
-      <c r="T28" s="20"/>
-      <c r="U28" s="20"/>
-    </row>
-    <row r="29" spans="1:24">
+      <c r="J28" s="26"/>
+      <c r="K28" s="26"/>
+      <c r="L28" s="26"/>
+      <c r="M28" s="26"/>
+      <c r="N28" s="26"/>
+      <c r="O28" s="26"/>
+      <c r="P28" s="26"/>
+      <c r="Q28" s="26"/>
+      <c r="R28" s="26"/>
+      <c r="S28" s="26"/>
+      <c r="T28" s="26"/>
+      <c r="U28" s="26"/>
+      <c r="V28" s="27"/>
+      <c r="AD28" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="29" spans="1:30">
       <c r="A29" s="11" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B29" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C29" s="11">
         <v>1</v>
@@ -3405,10 +3404,10 @@
         <v>1</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="H29" s="21">
         <v>46449</v>
@@ -3416,28 +3415,28 @@
       <c r="I29" s="21">
         <v>46363</v>
       </c>
-      <c r="J29" s="21"/>
-      <c r="K29" s="20"/>
-      <c r="L29" s="20"/>
-      <c r="M29" s="20"/>
-      <c r="N29" s="20"/>
-      <c r="O29" s="20"/>
-      <c r="P29" s="20"/>
-      <c r="Q29" s="20"/>
-      <c r="R29" s="20"/>
-      <c r="S29" s="20"/>
-      <c r="T29" s="20"/>
-      <c r="U29" s="20"/>
-      <c r="V29" s="20"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="26"/>
+      <c r="L29" s="26"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="26"/>
+      <c r="O29" s="26"/>
+      <c r="P29" s="26"/>
+      <c r="Q29" s="26"/>
+      <c r="R29" s="26"/>
+      <c r="S29" s="26"/>
+      <c r="T29" s="26"/>
+      <c r="U29" s="26"/>
+      <c r="V29" s="26"/>
       <c r="W29" s="20"/>
       <c r="X29" s="20"/>
     </row>
-    <row r="30" spans="1:24">
+    <row r="30" spans="1:30">
       <c r="A30" s="11" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B30" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C30" s="11">
         <v>1</v>
@@ -3446,13 +3445,13 @@
         <v>306</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="H30" s="21">
         <v>46449</v>
@@ -3460,25 +3459,26 @@
       <c r="I30" s="21">
         <v>46363</v>
       </c>
-      <c r="J30" s="21"/>
-      <c r="K30" s="20"/>
-      <c r="L30" s="20"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="20"/>
-      <c r="O30" s="20"/>
-      <c r="P30" s="20"/>
-      <c r="Q30" s="20"/>
-      <c r="R30" s="20"/>
-      <c r="S30" s="20"/>
-      <c r="T30" s="20"/>
-      <c r="U30" s="20"/>
-    </row>
-    <row r="31" spans="1:24">
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="26"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="26"/>
+      <c r="U30" s="26"/>
+      <c r="V30" s="27"/>
+    </row>
+    <row r="31" spans="1:30">
       <c r="A31" s="11" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C31" s="11">
         <v>3</v>
@@ -3490,10 +3490,10 @@
         <v>1</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="H31" s="21">
         <v>46449</v>
@@ -3501,25 +3501,26 @@
       <c r="I31" s="21">
         <v>46363</v>
       </c>
-      <c r="J31" s="21"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="20"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="20"/>
-      <c r="O31" s="20"/>
-      <c r="P31" s="20"/>
-      <c r="Q31" s="20"/>
-      <c r="R31" s="20"/>
-      <c r="S31" s="20"/>
-      <c r="T31" s="20"/>
-      <c r="U31" s="20"/>
-    </row>
-    <row r="32" spans="1:24">
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="26"/>
+      <c r="M31" s="26"/>
+      <c r="N31" s="26"/>
+      <c r="O31" s="26"/>
+      <c r="P31" s="26"/>
+      <c r="Q31" s="26"/>
+      <c r="R31" s="26"/>
+      <c r="S31" s="26"/>
+      <c r="T31" s="26"/>
+      <c r="U31" s="26"/>
+      <c r="V31" s="27"/>
+    </row>
+    <row r="32" spans="1:30">
       <c r="A32" s="11" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B32" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C32" s="11">
         <v>3</v>
@@ -3531,10 +3532,10 @@
         <v>2</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="H32" s="21">
         <v>46449</v>
@@ -3542,43 +3543,43 @@
       <c r="I32" s="21">
         <v>46363</v>
       </c>
-      <c r="J32" s="21"/>
-      <c r="K32" s="20"/>
-      <c r="L32" s="20"/>
-      <c r="M32" s="20"/>
-      <c r="N32" s="20"/>
-      <c r="O32" s="20"/>
-      <c r="P32" s="20"/>
-      <c r="Q32" s="20"/>
-      <c r="R32" s="20"/>
-      <c r="S32" s="20"/>
-      <c r="T32" s="20"/>
-      <c r="U32" s="20"/>
-      <c r="V32" s="20"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="26"/>
+      <c r="L32" s="26"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="26"/>
+      <c r="O32" s="26"/>
+      <c r="P32" s="26"/>
+      <c r="Q32" s="26"/>
+      <c r="R32" s="26"/>
+      <c r="S32" s="26"/>
+      <c r="T32" s="26"/>
+      <c r="U32" s="26"/>
+      <c r="V32" s="26"/>
       <c r="W32" s="20"/>
       <c r="X32" s="20"/>
     </row>
-    <row r="33" spans="1:24">
+    <row r="33" spans="1:30">
       <c r="A33" s="11" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D33" s="11">
         <v>16</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="H33" s="21">
         <v>46449</v>
@@ -3586,53 +3587,69 @@
       <c r="I33" s="21">
         <v>46363</v>
       </c>
-      <c r="J33" s="21">
+      <c r="J33" s="26">
         <v>46267</v>
       </c>
-      <c r="K33" s="20">
+      <c r="K33" s="26">
         <v>46273</v>
       </c>
-      <c r="L33" s="20">
+      <c r="L33" s="26">
         <v>46274</v>
       </c>
-      <c r="M33" s="20">
+      <c r="M33" s="26">
         <v>46293</v>
       </c>
-      <c r="N33" s="20">
+      <c r="N33" s="26">
         <v>46295</v>
       </c>
-      <c r="O33" s="20"/>
-      <c r="P33" s="20"/>
-      <c r="Q33" s="20"/>
-      <c r="R33" s="20"/>
-      <c r="S33" s="20"/>
-      <c r="T33" s="20"/>
-      <c r="U33" s="20"/>
-      <c r="V33" s="20"/>
+      <c r="O33" s="26">
+        <v>46295</v>
+      </c>
+      <c r="P33" s="26">
+        <v>46300</v>
+      </c>
+      <c r="Q33" s="26">
+        <v>46300</v>
+      </c>
+      <c r="R33" s="26">
+        <v>46301</v>
+      </c>
+      <c r="S33" s="26">
+        <v>46301</v>
+      </c>
+      <c r="T33" s="26">
+        <v>46303</v>
+      </c>
+      <c r="U33" s="26">
+        <v>46303</v>
+      </c>
+      <c r="V33" s="26">
+        <v>46309</v>
+      </c>
       <c r="W33" s="20"/>
       <c r="X33" s="20"/>
     </row>
-    <row r="34" spans="1:24">
+    <row r="34" spans="1:30">
       <c r="A34" s="11" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C34" s="11">
         <v>5</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="H34" s="21">
         <v>46449</v>
@@ -3640,21 +3657,26 @@
       <c r="I34" s="21">
         <v>46363</v>
       </c>
-      <c r="J34" s="21"/>
-      <c r="O34" s="20"/>
-      <c r="P34" s="20"/>
-      <c r="Q34" s="20"/>
-      <c r="R34" s="20"/>
-      <c r="S34" s="20"/>
-      <c r="T34" s="20"/>
-      <c r="U34" s="20"/>
-    </row>
-    <row r="35" spans="1:24">
+      <c r="J34" s="26"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="27"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="27"/>
+      <c r="O34" s="26"/>
+      <c r="P34" s="26"/>
+      <c r="Q34" s="26"/>
+      <c r="R34" s="26"/>
+      <c r="S34" s="26"/>
+      <c r="T34" s="26"/>
+      <c r="U34" s="26"/>
+      <c r="V34" s="27"/>
+    </row>
+    <row r="35" spans="1:30">
       <c r="A35" s="11" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C35" s="11">
         <v>6</v>
@@ -3666,10 +3688,10 @@
         <v>12</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H35" s="21">
         <v>46449</v>
@@ -3677,26 +3699,28 @@
       <c r="I35" s="21">
         <v>46363</v>
       </c>
-      <c r="J35" s="21"/>
-      <c r="K35" s="20"/>
-      <c r="L35" s="20"/>
-      <c r="O35" s="20"/>
-      <c r="P35" s="20"/>
-      <c r="Q35" s="20"/>
-      <c r="R35" s="20"/>
-      <c r="S35" s="20"/>
-      <c r="T35" s="20"/>
-      <c r="U35" s="20"/>
-      <c r="V35" s="20"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="26"/>
+      <c r="M35" s="27"/>
+      <c r="N35" s="27"/>
+      <c r="O35" s="26"/>
+      <c r="P35" s="26"/>
+      <c r="Q35" s="26"/>
+      <c r="R35" s="26"/>
+      <c r="S35" s="26"/>
+      <c r="T35" s="26"/>
+      <c r="U35" s="26"/>
+      <c r="V35" s="26"/>
       <c r="W35" s="20"/>
       <c r="X35" s="20"/>
     </row>
-    <row r="36" spans="1:24">
+    <row r="36" spans="1:30">
       <c r="A36" s="11" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C36" s="11">
         <v>7</v>
@@ -3708,10 +3732,10 @@
         <v>4</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="H36" s="21">
         <v>46449</v>
@@ -3719,37 +3743,41 @@
       <c r="I36" s="21">
         <v>46363</v>
       </c>
-      <c r="M36" s="20"/>
-      <c r="N36" s="20"/>
-      <c r="O36" s="20"/>
-      <c r="P36" s="20"/>
-      <c r="Q36" s="20"/>
-      <c r="R36" s="20"/>
-      <c r="S36" s="20"/>
-      <c r="T36" s="20"/>
-      <c r="U36" s="20"/>
-    </row>
-    <row r="37" spans="1:24">
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="26"/>
+      <c r="N36" s="26"/>
+      <c r="O36" s="26"/>
+      <c r="P36" s="26"/>
+      <c r="Q36" s="26"/>
+      <c r="R36" s="26"/>
+      <c r="S36" s="26"/>
+      <c r="T36" s="26"/>
+      <c r="U36" s="26"/>
+      <c r="V36" s="27"/>
+    </row>
+    <row r="37" spans="1:30">
       <c r="A37" s="11" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="C37" s="11">
         <v>8</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="G37" s="19" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="H37" s="21">
         <v>46449</v>
@@ -3757,25 +3785,28 @@
       <c r="I37" s="21">
         <v>46363</v>
       </c>
-      <c r="M37" s="20"/>
-      <c r="N37" s="20"/>
-      <c r="O37" s="20"/>
-      <c r="P37" s="20"/>
-      <c r="Q37" s="20"/>
-      <c r="R37" s="20"/>
-      <c r="S37" s="20"/>
-      <c r="T37" s="20"/>
-      <c r="U37" s="20"/>
-      <c r="V37" s="20"/>
+      <c r="J37" s="27"/>
+      <c r="K37" s="27"/>
+      <c r="L37" s="27"/>
+      <c r="M37" s="26"/>
+      <c r="N37" s="26"/>
+      <c r="O37" s="26"/>
+      <c r="P37" s="26"/>
+      <c r="Q37" s="26"/>
+      <c r="R37" s="26"/>
+      <c r="S37" s="26"/>
+      <c r="T37" s="26"/>
+      <c r="U37" s="26"/>
+      <c r="V37" s="26"/>
       <c r="W37" s="20"/>
       <c r="X37" s="20"/>
     </row>
-    <row r="38" spans="1:24">
+    <row r="38" spans="1:30">
       <c r="A38" s="11" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C38" s="11">
         <v>9</v>
@@ -3787,10 +3818,10 @@
         <v>2</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H38" s="21">
         <v>46449</v>
@@ -3798,35 +3829,43 @@
       <c r="I38" s="21">
         <v>46363</v>
       </c>
-      <c r="J38" s="21">
+      <c r="J38" s="26">
         <v>46281</v>
       </c>
-      <c r="K38" s="20">
+      <c r="K38" s="26">
         <v>46287</v>
       </c>
-      <c r="L38" s="20">
+      <c r="L38" s="26">
         <v>46289</v>
       </c>
-      <c r="M38" s="20">
+      <c r="M38" s="26">
         <v>46290</v>
       </c>
-      <c r="N38" s="20">
+      <c r="N38" s="26">
         <v>46293</v>
       </c>
-      <c r="O38" s="20"/>
-      <c r="P38" s="20"/>
-      <c r="Q38" s="20"/>
-      <c r="R38" s="20"/>
-      <c r="S38" s="20"/>
-      <c r="T38" s="20"/>
-      <c r="U38" s="20"/>
-    </row>
-    <row r="39" spans="1:24">
+      <c r="O38" s="26">
+        <v>46295</v>
+      </c>
+      <c r="P38" s="26">
+        <v>46295</v>
+      </c>
+      <c r="Q38" s="26"/>
+      <c r="R38" s="26"/>
+      <c r="S38" s="26"/>
+      <c r="T38" s="26"/>
+      <c r="U38" s="26"/>
+      <c r="V38" s="27"/>
+      <c r="AD38" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30">
       <c r="A39" s="11" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="C39" s="11">
         <v>10</v>
@@ -3835,13 +3874,13 @@
         <v>14</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="H39" s="21">
         <v>46449</v>
@@ -3849,43 +3888,43 @@
       <c r="I39" s="21">
         <v>46363</v>
       </c>
-      <c r="J39" s="21"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="20"/>
-      <c r="P39" s="20"/>
-      <c r="Q39" s="20"/>
-      <c r="R39" s="20"/>
-      <c r="S39" s="20"/>
-      <c r="T39" s="20"/>
-      <c r="U39" s="20"/>
-      <c r="V39" s="20"/>
+      <c r="J39" s="26"/>
+      <c r="K39" s="26"/>
+      <c r="L39" s="26"/>
+      <c r="M39" s="26"/>
+      <c r="N39" s="26"/>
+      <c r="O39" s="26"/>
+      <c r="P39" s="26"/>
+      <c r="Q39" s="26"/>
+      <c r="R39" s="26"/>
+      <c r="S39" s="26"/>
+      <c r="T39" s="26"/>
+      <c r="U39" s="26"/>
+      <c r="V39" s="26"/>
       <c r="W39" s="20"/>
       <c r="X39" s="20"/>
     </row>
-    <row r="40" spans="1:24">
+    <row r="40" spans="1:30">
       <c r="A40" s="11" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B40" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C40" s="11">
         <v>1</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="H40" s="21">
         <v>46491</v>
@@ -3893,25 +3932,26 @@
       <c r="I40" s="21">
         <v>46398</v>
       </c>
-      <c r="J40" s="21"/>
-      <c r="K40" s="20"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="20"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="20"/>
-      <c r="P40" s="20"/>
-      <c r="Q40" s="20"/>
-      <c r="R40" s="20"/>
-      <c r="S40" s="20"/>
-      <c r="T40" s="20"/>
-      <c r="U40" s="20"/>
-    </row>
-    <row r="41" spans="1:24">
+      <c r="J40" s="26"/>
+      <c r="K40" s="26"/>
+      <c r="L40" s="26"/>
+      <c r="M40" s="26"/>
+      <c r="N40" s="26"/>
+      <c r="O40" s="26"/>
+      <c r="P40" s="26"/>
+      <c r="Q40" s="26"/>
+      <c r="R40" s="26"/>
+      <c r="S40" s="26"/>
+      <c r="T40" s="26"/>
+      <c r="U40" s="26"/>
+      <c r="V40" s="27"/>
+    </row>
+    <row r="41" spans="1:30">
       <c r="A41" s="11" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B41" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C41" s="11">
         <v>1</v>
@@ -3920,13 +3960,13 @@
         <v>284</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="H41" s="21">
         <v>46491</v>
@@ -3934,28 +3974,28 @@
       <c r="I41" s="21">
         <v>46398</v>
       </c>
-      <c r="J41" s="21"/>
-      <c r="K41" s="20"/>
-      <c r="L41" s="20"/>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="20"/>
-      <c r="Q41" s="20"/>
-      <c r="R41" s="20"/>
-      <c r="S41" s="20"/>
-      <c r="T41" s="20"/>
-      <c r="U41" s="20"/>
-      <c r="V41" s="20"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="26"/>
+      <c r="L41" s="26"/>
+      <c r="M41" s="26"/>
+      <c r="N41" s="26"/>
+      <c r="O41" s="26"/>
+      <c r="P41" s="26"/>
+      <c r="Q41" s="26"/>
+      <c r="R41" s="26"/>
+      <c r="S41" s="26"/>
+      <c r="T41" s="26"/>
+      <c r="U41" s="26"/>
+      <c r="V41" s="26"/>
       <c r="W41" s="20"/>
       <c r="X41" s="20"/>
     </row>
-    <row r="42" spans="1:24">
+    <row r="42" spans="1:30">
       <c r="A42" s="11" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B42" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C42" s="11">
         <v>1</v>
@@ -3967,10 +4007,10 @@
         <v>6</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="H42" s="21">
         <v>46491</v>
@@ -3991,12 +4031,12 @@
       <c r="T42" s="20"/>
       <c r="U42" s="20"/>
     </row>
-    <row r="43" spans="1:24">
+    <row r="43" spans="1:30">
       <c r="A43" s="11" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="B43" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C43" s="11">
         <v>2</v>
@@ -4005,13 +4045,13 @@
         <v>167</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="H43" s="21">
         <v>46491</v>
@@ -4035,12 +4075,12 @@
       <c r="W43" s="20"/>
       <c r="X43" s="20"/>
     </row>
-    <row r="44" spans="1:24">
+    <row r="44" spans="1:30">
       <c r="A44" s="11" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B44" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C44" s="11">
         <v>4</v>
@@ -4052,10 +4092,10 @@
         <v>2</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="H44" s="21">
         <v>46491</v>
@@ -4079,12 +4119,12 @@
       <c r="W44" s="20"/>
       <c r="X44" s="20"/>
     </row>
-    <row r="45" spans="1:24">
+    <row r="45" spans="1:30">
       <c r="A45" s="11" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C45" s="11">
         <v>5</v>
@@ -4096,10 +4136,10 @@
         <v>12</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="H45" s="21">
         <v>46491</v>
@@ -4120,12 +4160,12 @@
       <c r="T45" s="20"/>
       <c r="U45" s="20"/>
     </row>
-    <row r="46" spans="1:24">
+    <row r="46" spans="1:30">
       <c r="A46" s="11" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B46" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C46" s="11">
         <v>6</v>
@@ -4137,10 +4177,10 @@
         <v>12</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="H46" s="21">
         <v>46491</v>
@@ -4164,27 +4204,27 @@
       <c r="W46" s="20"/>
       <c r="X46" s="20"/>
     </row>
-    <row r="47" spans="1:24">
+    <row r="47" spans="1:30">
       <c r="A47" s="11" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B47" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C47" s="11">
         <v>7</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="H47" s="21">
         <v>46491</v>
@@ -4205,12 +4245,12 @@
       <c r="T47" s="20"/>
       <c r="U47" s="20"/>
     </row>
-    <row r="48" spans="1:24">
+    <row r="48" spans="1:30">
       <c r="A48" s="11" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="B48" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="C48" s="11">
         <v>9</v>
@@ -4219,13 +4259,13 @@
         <v>65</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="F48" s="19" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="G48" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H48" s="21">
         <v>46491</v>
@@ -4251,10 +4291,10 @@
     </row>
     <row r="49" spans="1:24">
       <c r="A49" s="11" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B49" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C49" s="11">
         <v>10</v>
@@ -4266,10 +4306,10 @@
         <v>6</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="G49" s="19" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="H49" s="21">
         <v>46491</v>
@@ -4292,10 +4332,10 @@
     </row>
     <row r="50" spans="1:24">
       <c r="A50" s="11" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="B50" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="C50" s="11">
         <v>2</v>
@@ -4307,10 +4347,10 @@
         <v>0</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="H50" s="21">
         <v>46526</v>
@@ -4333,10 +4373,10 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" s="11" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B51" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="C51" s="11">
         <v>3</v>
@@ -4348,10 +4388,10 @@
         <v>4</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="H51" s="21">
         <v>46526</v>
@@ -4377,10 +4417,10 @@
     </row>
     <row r="52" spans="1:24">
       <c r="A52" s="11" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="B52" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="C52" s="11">
         <v>5</v>
@@ -4392,10 +4432,10 @@
         <v>0</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="H52" s="21">
         <v>46526</v>
@@ -4421,10 +4461,10 @@
     </row>
     <row r="53" spans="1:24">
       <c r="A53" s="11" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="B53" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="C53" s="11">
         <v>6</v>
@@ -4436,10 +4476,10 @@
         <v>10</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="G53" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H53" s="21">
         <v>46526</v>
@@ -4462,10 +4502,10 @@
     </row>
     <row r="54" spans="1:24">
       <c r="A54" s="11" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="B54" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="C54" s="11">
         <v>7</v>
@@ -4477,10 +4517,10 @@
         <v>1</v>
       </c>
       <c r="F54" s="19" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="G54" s="19" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="H54" s="21">
         <v>46526</v>
@@ -4503,10 +4543,10 @@
     </row>
     <row r="55" spans="1:24">
       <c r="A55" s="11" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="B55" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C55" s="11">
         <v>9</v>
@@ -4518,10 +4558,10 @@
         <v>19</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="H55" s="21">
         <v>46526</v>
@@ -4547,10 +4587,10 @@
     </row>
     <row r="56" spans="1:24">
       <c r="A56" s="11" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B56" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C56" s="11">
         <v>9</v>
@@ -4559,13 +4599,13 @@
         <v>65</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="F56" s="19" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="G56" s="19" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="H56" s="21">
         <v>46526</v>
@@ -4591,10 +4631,10 @@
     </row>
     <row r="57" spans="1:24">
       <c r="A57" s="11" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B57" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C57" s="11">
         <v>10</v>
@@ -4603,13 +4643,13 @@
         <v>49</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F57" s="19" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="G57" s="19" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="H57" s="21">
         <v>46526</v>
@@ -4635,10 +4675,10 @@
     </row>
     <row r="58" spans="1:24">
       <c r="A58" s="23" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B58" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C58" s="11">
         <v>9</v>
@@ -4650,10 +4690,10 @@
         <v>1</v>
       </c>
       <c r="F58" s="19" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="G58" s="19" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="H58" s="21">
         <v>46526</v>
@@ -4685,7 +4725,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4697,19 +4737,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="34.049999999999997" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1">
@@ -5011,111 +5051,6 @@
         <v>32</v>
       </c>
       <c r="E21" s="13"/>
-    </row>
-    <row r="22" spans="1:5" ht="21" customHeight="1">
-      <c r="A22" s="12">
-        <v>21</v>
-      </c>
-      <c r="B22" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="13"/>
-    </row>
-    <row r="23" spans="1:5" ht="21" customHeight="1">
-      <c r="A23" s="12">
-        <v>22</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" s="13"/>
-    </row>
-    <row r="24" spans="1:5" ht="21" customHeight="1">
-      <c r="A24" s="12">
-        <v>23</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" s="13"/>
-    </row>
-    <row r="25" spans="1:5" ht="21" customHeight="1">
-      <c r="A25" s="12">
-        <v>24</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E25" s="13"/>
-    </row>
-    <row r="26" spans="1:5" ht="21" customHeight="1">
-      <c r="A26" s="12">
-        <v>25</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="13"/>
-    </row>
-    <row r="27" spans="1:5" ht="21" customHeight="1">
-      <c r="A27" s="12">
-        <v>26</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="13"/>
-    </row>
-    <row r="28" spans="1:5" ht="21" customHeight="1">
-      <c r="A28" s="12">
-        <v>27</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Major Update on PPP 2027 on 10.20.26
</commit_message>
<xml_diff>
--- a/data/PPP-2027-Review-Tracking.xlsx
+++ b/data/PPP-2027-Review-Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ashtd-my.sharepoint.com/personal/niwesh_koirala_ardot_gov/Documents/Desktop/Github/PPP-2027-Review-Control-Center/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{908BCBEC-4003-4C53-A1F3-237188509867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{147AD658-2F46-437E-96AF-C7EB2A4CE2FE}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{908BCBEC-4003-4C53-A1F3-237188509867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9689658-65E4-4BBD-B618-228A6D0A7F6E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="675" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -549,9 +549,6 @@
     <t>Mill &amp; Overlay</t>
   </si>
   <si>
-    <t xml:space="preserve">2" Overlay; Add 2' Shoulders </t>
-  </si>
-  <si>
     <t>2" Mill &amp; 1.5" Overlay</t>
   </si>
   <si>
@@ -844,6 +841,9 @@
   </si>
   <si>
     <t>Send for DE Signature</t>
+  </si>
+  <si>
+    <t>FDR (Sec. 21 LM 4.665-9.802 &amp; Sec. 22 LM 0-1.92); Level Up &amp; 2” Overlay (Sec. 21 LM 9.802-14.586 &amp; Sec. 22 LM 1.92-7.715); Mill &amp; Overlay (Sec. 21 LM 14.586-16.848)</t>
   </si>
 </sst>
 </file>
@@ -1401,7 +1401,7 @@
     <col min="3" max="3" width="10" style="11" customWidth="1"/>
     <col min="4" max="5" width="12" style="11" customWidth="1"/>
     <col min="6" max="6" width="19.8984375" style="11" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19" style="11" customWidth="1"/>
+    <col min="7" max="7" width="98.69921875" style="11" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="14" style="11" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="18" style="11" customWidth="1"/>
@@ -2394,7 +2394,7 @@
         <v>46286</v>
       </c>
       <c r="AB11" s="24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AC11" s="20">
         <v>46294</v>
@@ -2753,8 +2753,11 @@
       <c r="AA15" s="24">
         <v>46308</v>
       </c>
+      <c r="AB15" s="20">
+        <v>46314</v>
+      </c>
       <c r="AD15" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="16" spans="1:30">
@@ -2774,7 +2777,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G16" s="19" t="s">
         <v>170</v>
@@ -2796,7 +2799,7 @@
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
       <c r="AD16" s="20" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:30">
@@ -2816,7 +2819,7 @@
         <v>2</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G17" s="19" t="s">
         <v>158</v>
@@ -2841,7 +2844,7 @@
       <c r="W17" s="20"/>
       <c r="X17" s="20"/>
       <c r="AD17" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" spans="1:30">
@@ -2858,13 +2861,13 @@
         <v>65</v>
       </c>
       <c r="E18" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="F18" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="F18" s="19" t="s">
-        <v>200</v>
-      </c>
       <c r="G18" s="19" t="s">
-        <v>171</v>
+        <v>269</v>
       </c>
       <c r="H18" s="21">
         <v>46407</v>
@@ -2886,7 +2889,7 @@
       <c r="U18" s="26"/>
       <c r="V18" s="27"/>
       <c r="AD18" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:30">
@@ -2903,13 +2906,13 @@
         <v>27</v>
       </c>
       <c r="E19" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="F19" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="F19" s="19" t="s">
-        <v>202</v>
-      </c>
       <c r="G19" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H19" s="21">
         <v>46407</v>
@@ -2933,7 +2936,7 @@
       <c r="W19" s="20"/>
       <c r="X19" s="20"/>
       <c r="AD19" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:30">
@@ -2953,10 +2956,10 @@
         <v>1</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H20" s="21">
         <v>46407</v>
@@ -2978,7 +2981,7 @@
       <c r="U20" s="26"/>
       <c r="V20" s="27"/>
       <c r="AD20" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:30">
@@ -2998,10 +3001,10 @@
         <v>1</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H21" s="21">
         <v>46407</v>
@@ -3025,7 +3028,7 @@
       <c r="W21" s="20"/>
       <c r="X21" s="20"/>
       <c r="AD21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:30">
@@ -3045,10 +3048,10 @@
         <v>15</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H22" s="21">
         <v>46407</v>
@@ -3074,9 +3077,10 @@
       <c r="S22" s="26"/>
       <c r="T22" s="26"/>
       <c r="U22" s="26"/>
-      <c r="V22" s="27"/>
+      <c r="V22" s="26"/>
+      <c r="W22" s="20"/>
       <c r="AD22" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:30">
@@ -3093,13 +3097,13 @@
         <v>14</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>67</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H23" s="21">
         <v>46407</v>
@@ -3123,7 +3127,7 @@
       <c r="W23" s="20"/>
       <c r="X23" s="20"/>
       <c r="AD23" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="24" spans="1:30">
@@ -3140,13 +3144,13 @@
         <v>175</v>
       </c>
       <c r="E24" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="F24" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="F24" s="19" t="s">
-        <v>208</v>
-      </c>
       <c r="G24" s="19" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H24" s="21">
         <v>46407</v>
@@ -3154,9 +3158,15 @@
       <c r="I24" s="21">
         <v>46321</v>
       </c>
-      <c r="J24" s="26"/>
-      <c r="K24" s="26"/>
-      <c r="L24" s="26"/>
+      <c r="J24" s="26">
+        <v>46309</v>
+      </c>
+      <c r="K24" s="26">
+        <v>46314</v>
+      </c>
+      <c r="L24" s="26">
+        <v>46314</v>
+      </c>
       <c r="M24" s="26"/>
       <c r="N24" s="26"/>
       <c r="O24" s="27"/>
@@ -3166,9 +3176,10 @@
       <c r="S24" s="26"/>
       <c r="T24" s="26"/>
       <c r="U24" s="26"/>
-      <c r="V24" s="27"/>
+      <c r="V24" s="26"/>
+      <c r="W24" s="20"/>
       <c r="AD24" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="25" spans="1:30">
@@ -3185,13 +3196,13 @@
         <v>13</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H25" s="21">
         <v>46407</v>
@@ -3215,7 +3226,7 @@
       <c r="W25" s="20"/>
       <c r="X25" s="20"/>
       <c r="AD25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="26" spans="1:30">
@@ -3238,7 +3249,7 @@
         <v>73</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H26" s="21">
         <v>46407</v>
@@ -3273,12 +3284,23 @@
       <c r="R26" s="26">
         <v>46308</v>
       </c>
-      <c r="S26" s="26"/>
-      <c r="T26" s="26"/>
-      <c r="U26" s="26"/>
-      <c r="V26" s="27"/>
+      <c r="S26" s="26">
+        <v>46309</v>
+      </c>
+      <c r="T26" s="26">
+        <v>46309</v>
+      </c>
+      <c r="U26" s="26">
+        <v>46309</v>
+      </c>
+      <c r="V26" s="26">
+        <v>46309</v>
+      </c>
+      <c r="W26" s="20">
+        <v>46311</v>
+      </c>
       <c r="AD26" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:30">
@@ -3298,7 +3320,7 @@
         <v>3</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G27" s="19" t="s">
         <v>164</v>
@@ -3330,8 +3352,12 @@
       <c r="P27" s="26">
         <v>46295</v>
       </c>
-      <c r="Q27" s="26"/>
-      <c r="R27" s="26"/>
+      <c r="Q27" s="26">
+        <v>46309</v>
+      </c>
+      <c r="R27" s="26">
+        <v>46309</v>
+      </c>
       <c r="S27" s="26"/>
       <c r="T27" s="26"/>
       <c r="U27" s="26"/>
@@ -3339,7 +3365,7 @@
       <c r="W27" s="20"/>
       <c r="X27" s="20"/>
       <c r="AD27" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="28" spans="1:30">
@@ -3356,13 +3382,13 @@
         <v>49</v>
       </c>
       <c r="E28" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="F28" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="F28" s="19" t="s">
-        <v>212</v>
-      </c>
       <c r="G28" s="19" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H28" s="21">
         <v>46407</v>
@@ -3370,21 +3396,28 @@
       <c r="I28" s="21">
         <v>46321</v>
       </c>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="26"/>
+      <c r="J28" s="26">
+        <v>46309</v>
+      </c>
+      <c r="K28" s="26">
+        <v>46314</v>
+      </c>
+      <c r="L28" s="26">
+        <v>46314</v>
+      </c>
+      <c r="M28" s="27"/>
       <c r="N28" s="26"/>
-      <c r="O28" s="26"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="26"/>
-      <c r="S28" s="26"/>
-      <c r="T28" s="26"/>
-      <c r="U28" s="26"/>
+      <c r="O28" s="27"/>
+      <c r="P28" s="27"/>
+      <c r="Q28" s="27"/>
+      <c r="R28" s="27"/>
+      <c r="S28" s="27"/>
+      <c r="T28" s="27"/>
+      <c r="U28" s="27"/>
       <c r="V28" s="27"/>
+      <c r="W28" s="20"/>
       <c r="AD28" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="29" spans="1:30">
@@ -3404,10 +3437,10 @@
         <v>1</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H29" s="21">
         <v>46449</v>
@@ -3445,13 +3478,13 @@
         <v>306</v>
       </c>
       <c r="E30" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="H30" s="21">
         <v>46449</v>
@@ -3490,10 +3523,10 @@
         <v>1</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H31" s="21">
         <v>46449</v>
@@ -3532,10 +3565,10 @@
         <v>2</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H32" s="21">
         <v>46449</v>
@@ -3573,13 +3606,13 @@
         <v>16</v>
       </c>
       <c r="E33" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="F33" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="F33" s="19" t="s">
-        <v>217</v>
-      </c>
       <c r="G33" s="19" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H33" s="21">
         <v>46449</v>
@@ -3640,16 +3673,16 @@
         <v>5</v>
       </c>
       <c r="D34" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="E34" s="11" t="s">
         <v>218</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="F34" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="F34" s="19" t="s">
-        <v>220</v>
-      </c>
       <c r="G34" s="19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H34" s="21">
         <v>46449</v>
@@ -3662,14 +3695,14 @@
       <c r="L34" s="27"/>
       <c r="M34" s="27"/>
       <c r="N34" s="27"/>
-      <c r="O34" s="26"/>
+      <c r="O34" s="27"/>
       <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="26"/>
-      <c r="V34" s="27"/>
+      <c r="Q34" s="27"/>
+      <c r="R34" s="27"/>
+      <c r="S34" s="27"/>
+      <c r="T34" s="27"/>
+      <c r="U34" s="27"/>
+      <c r="V34" s="26"/>
     </row>
     <row r="35" spans="1:30">
       <c r="A35" s="11" t="s">
@@ -3688,7 +3721,7 @@
         <v>12</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G35" s="19" t="s">
         <v>164</v>
@@ -3704,13 +3737,13 @@
       <c r="L35" s="26"/>
       <c r="M35" s="27"/>
       <c r="N35" s="27"/>
-      <c r="O35" s="26"/>
-      <c r="P35" s="26"/>
-      <c r="Q35" s="26"/>
-      <c r="R35" s="26"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="26"/>
-      <c r="U35" s="26"/>
+      <c r="O35" s="27"/>
+      <c r="P35" s="27"/>
+      <c r="Q35" s="27"/>
+      <c r="R35" s="27"/>
+      <c r="S35" s="27"/>
+      <c r="T35" s="27"/>
+      <c r="U35" s="27"/>
       <c r="V35" s="26"/>
       <c r="W35" s="20"/>
       <c r="X35" s="20"/>
@@ -3732,10 +3765,10 @@
         <v>4</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H36" s="21">
         <v>46449</v>
@@ -3748,14 +3781,14 @@
       <c r="L36" s="27"/>
       <c r="M36" s="26"/>
       <c r="N36" s="26"/>
-      <c r="O36" s="26"/>
-      <c r="P36" s="26"/>
-      <c r="Q36" s="26"/>
-      <c r="R36" s="26"/>
-      <c r="S36" s="26"/>
-      <c r="T36" s="26"/>
-      <c r="U36" s="26"/>
-      <c r="V36" s="27"/>
+      <c r="O36" s="27"/>
+      <c r="P36" s="27"/>
+      <c r="Q36" s="27"/>
+      <c r="R36" s="27"/>
+      <c r="S36" s="27"/>
+      <c r="T36" s="27"/>
+      <c r="U36" s="27"/>
+      <c r="V36" s="26"/>
     </row>
     <row r="37" spans="1:30">
       <c r="A37" s="11" t="s">
@@ -3768,16 +3801,16 @@
         <v>8</v>
       </c>
       <c r="D37" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="E37" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="E37" s="11" t="s">
+      <c r="F37" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="F37" s="19" t="s">
-        <v>225</v>
-      </c>
       <c r="G37" s="19" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H37" s="21">
         <v>46449</v>
@@ -3790,13 +3823,13 @@
       <c r="L37" s="27"/>
       <c r="M37" s="26"/>
       <c r="N37" s="26"/>
-      <c r="O37" s="26"/>
-      <c r="P37" s="26"/>
-      <c r="Q37" s="26"/>
+      <c r="O37" s="27"/>
+      <c r="P37" s="27"/>
+      <c r="Q37" s="27"/>
       <c r="R37" s="26"/>
-      <c r="S37" s="26"/>
-      <c r="T37" s="26"/>
-      <c r="U37" s="26"/>
+      <c r="S37" s="27"/>
+      <c r="T37" s="27"/>
+      <c r="U37" s="27"/>
       <c r="V37" s="26"/>
       <c r="W37" s="20"/>
       <c r="X37" s="20"/>
@@ -3818,7 +3851,7 @@
         <v>2</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G38" s="19" t="s">
         <v>164</v>
@@ -3850,14 +3883,22 @@
       <c r="P38" s="26">
         <v>46295</v>
       </c>
-      <c r="Q38" s="26"/>
-      <c r="R38" s="26"/>
-      <c r="S38" s="26"/>
-      <c r="T38" s="26"/>
-      <c r="U38" s="26"/>
-      <c r="V38" s="27"/>
+      <c r="Q38" s="26">
+        <v>46308</v>
+      </c>
+      <c r="R38" s="26">
+        <v>45578</v>
+      </c>
+      <c r="S38" s="26">
+        <v>46311</v>
+      </c>
+      <c r="T38" s="26">
+        <v>46311</v>
+      </c>
+      <c r="U38" s="27"/>
+      <c r="V38" s="26"/>
       <c r="AD38" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:30">
@@ -3874,13 +3915,13 @@
         <v>14</v>
       </c>
       <c r="E39" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="F39" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="F39" s="19" t="s">
-        <v>228</v>
-      </c>
       <c r="G39" s="19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H39" s="21">
         <v>46449</v>
@@ -3915,16 +3956,16 @@
         <v>1</v>
       </c>
       <c r="D40" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="E40" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="E40" s="11" t="s">
-        <v>230</v>
-      </c>
       <c r="F40" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H40" s="21">
         <v>46491</v>
@@ -3960,13 +4001,13 @@
         <v>284</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H41" s="21">
         <v>46491</v>
@@ -4007,10 +4048,10 @@
         <v>6</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G42" s="19" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H42" s="21">
         <v>46491</v>
@@ -4033,10 +4074,10 @@
     </row>
     <row r="43" spans="1:30">
       <c r="A43" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B43" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C43" s="11">
         <v>2</v>
@@ -4045,13 +4086,13 @@
         <v>167</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H43" s="21">
         <v>46491</v>
@@ -4092,10 +4133,10 @@
         <v>2</v>
       </c>
       <c r="F44" s="19" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H44" s="21">
         <v>46491</v>
@@ -4136,10 +4177,10 @@
         <v>12</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H45" s="21">
         <v>46491</v>
@@ -4180,7 +4221,7 @@
         <v>69</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H46" s="21">
         <v>46491</v>
@@ -4215,16 +4256,16 @@
         <v>7</v>
       </c>
       <c r="D47" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="E47" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="E47" s="11" t="s">
+      <c r="F47" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="F47" s="19" t="s">
-        <v>235</v>
-      </c>
       <c r="G47" s="19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H47" s="21">
         <v>46491</v>
@@ -4259,10 +4300,10 @@
         <v>65</v>
       </c>
       <c r="E48" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="F48" s="19" t="s">
         <v>236</v>
-      </c>
-      <c r="F48" s="19" t="s">
-        <v>237</v>
       </c>
       <c r="G48" s="19" t="s">
         <v>164</v>
@@ -4306,10 +4347,10 @@
         <v>6</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G49" s="19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H49" s="21">
         <v>46491</v>
@@ -4332,10 +4373,10 @@
     </row>
     <row r="50" spans="1:24">
       <c r="A50" s="11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B50" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C50" s="11">
         <v>2</v>
@@ -4347,7 +4388,7 @@
         <v>0</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G50" s="19" t="s">
         <v>170</v>
@@ -4373,10 +4414,10 @@
     </row>
     <row r="51" spans="1:24">
       <c r="A51" s="11" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B51" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C51" s="11">
         <v>3</v>
@@ -4388,7 +4429,7 @@
         <v>4</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G51" s="19" t="s">
         <v>168</v>
@@ -4435,7 +4476,7 @@
         <v>65</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H52" s="21">
         <v>46526</v>
@@ -4461,10 +4502,10 @@
     </row>
     <row r="53" spans="1:24">
       <c r="A53" s="11" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B53" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C53" s="11">
         <v>6</v>
@@ -4476,7 +4517,7 @@
         <v>10</v>
       </c>
       <c r="F53" s="19" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G53" s="19" t="s">
         <v>164</v>
@@ -4502,10 +4543,10 @@
     </row>
     <row r="54" spans="1:24">
       <c r="A54" s="11" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B54" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C54" s="11">
         <v>7</v>
@@ -4543,10 +4584,10 @@
     </row>
     <row r="55" spans="1:24">
       <c r="A55" s="11" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B55" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C55" s="11">
         <v>9</v>
@@ -4558,10 +4599,10 @@
         <v>19</v>
       </c>
       <c r="F55" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G55" s="19" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H55" s="21">
         <v>46526</v>
@@ -4599,10 +4640,10 @@
         <v>65</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F56" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G56" s="19" t="s">
         <v>170</v>
@@ -4643,13 +4684,13 @@
         <v>49</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F57" s="19" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G57" s="19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H57" s="21">
         <v>46526</v>
@@ -4675,10 +4716,10 @@
     </row>
     <row r="58" spans="1:24">
       <c r="A58" s="23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B58" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C58" s="11">
         <v>9</v>
@@ -4690,7 +4731,7 @@
         <v>1</v>
       </c>
       <c r="F58" s="19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G58" s="19" t="s">
         <v>164</v>

</xml_diff>